<commit_message>
Make TODO.md the only todo list, remove todo.txt, point the xlsx Todo sheet to it
</commit_message>
<xml_diff>
--- a/AmbermoonAdvanced.xlsx
+++ b/AmbermoonAdvanced.xlsx
@@ -20937,495 +20937,14 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:B119"/>
+  <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B2" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B4" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="4" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" s="4"/>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" s="4" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A17" s="10" t="s">
-        <v>2267</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A18" s="10" t="s">
-        <v>2268</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A19" s="10" t="s">
-        <v>2265</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A20" s="10" t="s">
-        <v>2266</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A21" s="10" t="s">
-        <v>2228</v>
-      </c>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A22" s="10" t="s">
-        <v>2229</v>
-      </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A23" s="10" t="s">
-        <v>2226</v>
-      </c>
-    </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A30" s="68" t="s">
-        <v>2225</v>
-      </c>
-    </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A31" s="68" t="s">
-        <v>2227</v>
-      </c>
-    </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A32" s="68" t="s">
-        <v>2263</v>
-      </c>
-    </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A36" s="68" t="s">
-        <v>2260</v>
-      </c>
-    </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A44" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A45" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A46" s="68" t="s">
-        <v>2269</v>
-      </c>
-    </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A47" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A48" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A49" s="68" t="s">
-        <v>2264</v>
-      </c>
-    </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A51" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A52" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A53" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A54" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A55" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A56" s="4" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="57" spans="1:1" ht="13.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A57" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="58" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A58" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A59" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="61" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A61" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="62" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A62" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="63" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A63" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="64" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A64" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A65" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="66" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A66" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A67" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="68" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A68" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="69" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A69" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="70" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A70" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="72" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A72" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="73" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A73" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="74" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A74" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="76" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A76" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="78" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A78" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="79" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A79" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="82" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A82" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="83" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A83" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="84" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A84" s="4" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="85" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A85" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="86" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A86" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="87" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A87" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="88" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A88" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="90" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A90" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="91" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A91" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="92" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A92" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="93" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A93" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="94" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A94" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="95" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A95" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="96" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A96" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="98" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A98" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="100" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A100" s="4" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="101" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A101" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="102" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A102" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="103" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A103" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="104" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A104" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="105" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A105" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="106" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A106" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="107" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A107" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="108" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A108" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="109" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A109" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="110" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A110" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="111" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A111" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="112" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A112" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="113" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A113" s="68" t="s">
-        <v>2270</v>
-      </c>
-    </row>
-    <row r="114" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A114" s="82" t="s">
-        <v>2271</v>
-      </c>
-    </row>
-    <row r="116" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A116" s="4" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="118" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A118" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="119" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A119" t="s">
-        <v>127</v>
+    <row r="1" spans="1:1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Die Todo-Liste steht jetzt in TODO.md im Repo (Ambermoon-Advanced, Branch episode4). Die Punkte dieses Blatts wurden dorthin übernommen.</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Unique goto point bits for Dor Grestin and the Spannenberg gardening shed, fix flags of english map 372
- Dor Grestin (339): SOUTH EXIT, NORTH EXIT, THE NEST and FOODSTUFFS used the bits 67-70 like goto
  points of the Rogue's wine cellar (265) and Spannenberg (263) (Ambermoon #99). The original now
  uses 79-82, which are taken in Advanced, so they use 103-106.
- Spannenberg (263): the new goto point at (17,23) used bit 16 like CITY PARK E, it now uses 17.
- English map 372 (Ship's End) had the flags 0x805a instead of 0x085a: magic was disabled and the
  internal shared map data flag was set.
- Documented in the GotoPoints sheet of the xlsx.
</commit_message>
<xml_diff>
--- a/AmbermoonAdvanced.xlsx
+++ b/AmbermoonAdvanced.xlsx
@@ -23516,7 +23516,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:A29"/>
+  <dimension ref="A1:A39"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="65.42578125" customWidth="1"/>
@@ -23660,6 +23660,62 @@
     <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>474</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">103: Ausgang Süd / South Exit (Dor Grestin) – war 67 (doppelt mit Ausgang im Weinkeller)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" spans="1:1">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">104: Ausgang Nord / North Exit (Dor Grestin) – war 68 (doppelt mit Training im Weinkeller)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" spans="1:1">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">105: Das Nest / The Nest (Dor Grestin) – war 69 (doppelt mit Gildenhändler im Weinkeller)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" spans="1:1">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">106: Lebensmittel / Foodstuffs (Dor Grestin) – war 70 (doppelt mit Stadthaus 1 in Spannenberg)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" spans="1:1">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hinweise (14.10.2026):</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" spans="1:1">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">- Dor Grestin: Die 4 Goto-Points oben nutzten schon im Original die Bits 67-70 doppelt (Ambermoon #99). Das Original nutzt jetzt 79-82, die in Advanced belegt sind, daher hier 103-106.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" spans="1:1">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">- 17: Der neue Spannenberg-Goto bei (17,23) "Parkverwaltung / Gardening Shed" nutzte fälschlich Bit 16 (wie Stadtgarten O) und nutzt jetzt 17.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" spans="1:1">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">- 101/102: In den Daten hat "Weiser / Wise Man" (S'Angrila) Bit 101. Ein Versteck-Goto existiert noch nicht. Frei sind 0 und 102, ab 107 ist alles frei.</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add the hideout goto point in S'Angrila (bit 102), update the goto point docs
- New goto point VERSTECK on map 441 at (27,24), in front of the dark house which leads to the
  hideout. It uses bit 102, the next free one (the wise man already uses 101).
- GotoPoints sheet: 17 is the park administration / gardening shed, 101 the wise man, 102 the
  hideout.
</commit_message>
<xml_diff>
--- a/AmbermoonAdvanced.xlsx
+++ b/AmbermoonAdvanced.xlsx
@@ -23538,8 +23538,10 @@
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>450</v>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">17: Parkverwaltung / Gardening Shed (Spannenberg)</t>
+        </is>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
@@ -23653,13 +23655,17 @@
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>473</v>
+      <c r="A28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">101: Weiser / Wise Man (S’Angrila)</t>
+        </is>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>474</v>
+      <c r="A29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">102: Versteck / Hideout (S’Angrila) – vor dem Dunklen Haus (27,24)</t>
+        </is>
       </c>
     </row>
     <row r="31" spans="1:1">
@@ -23707,14 +23713,14 @@
     <row r="38" spans="1:1">
       <c r="A38" t="inlineStr">
         <is>
-          <t xml:space="preserve">- 17: Der neue Spannenberg-Goto bei (17,23) "Parkverwaltung / Gardening Shed" nutzte fälschlich Bit 16 (wie Stadtgarten O) und nutzt jetzt 17.</t>
+          <t xml:space="preserve">- 17: Parkverwaltung / Gardening Shed (Spannenberg, bei (17,23)) nutzte fälschlich Bit 16 (wie Stadtgarten O) und nutzt jetzt 17.</t>
         </is>
       </c>
     </row>
     <row r="39" spans="1:1">
       <c r="A39" t="inlineStr">
         <is>
-          <t xml:space="preserve">- 101/102: In den Daten hat "Weiser / Wise Man" (S'Angrila) Bit 101. Ein Versteck-Goto existiert noch nicht. Frei sind 0 und 102, ab 107 ist alles frei.</t>
+          <t xml:space="preserve">- 101/102: Der Weise hatte in den Daten schon 101 statt wie geplant 102. Das Versteck hat jetzt 102. Bit 0 ist wie im Original unbenutzt, ab 107 ist alles frei.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rename the hideout goto point to Dunkles Haus / Dark House, use the name Gärtnerei in the data
- Goto point 102 in S'Angrila is called DUNKLES HAUS / DARK HOUSE to not spoil the hideout.
- The Spannenberg goto point 17 is GÄRTNEREI in AllTexts, the binary still had PARKVERWALTUNG.
  Its AllTexts file was latin-1 instead of UTF-8.
- GotoPoints sheet updated.
</commit_message>
<xml_diff>
--- a/AmbermoonAdvanced.xlsx
+++ b/AmbermoonAdvanced.xlsx
@@ -23540,7 +23540,7 @@
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">17: Parkverwaltung / Gardening Shed (Spannenberg)</t>
+          <t xml:space="preserve">17: Gärtnerei / Gardening Shed (Spannenberg)</t>
         </is>
       </c>
     </row>
@@ -23664,7 +23664,7 @@
     <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" t="inlineStr">
         <is>
-          <t xml:space="preserve">102: Versteck / Hideout (S’Angrila) – vor dem Dunklen Haus (27,24)</t>
+          <t xml:space="preserve">102: Dunkles Haus / Dark House (S’Angrila) – Eingang zum Versteck, (27,24)</t>
         </is>
       </c>
     </row>
@@ -23713,14 +23713,14 @@
     <row r="38" spans="1:1">
       <c r="A38" t="inlineStr">
         <is>
-          <t xml:space="preserve">- 17: Parkverwaltung / Gardening Shed (Spannenberg, bei (17,23)) nutzte fälschlich Bit 16 (wie Stadtgarten O) und nutzt jetzt 17.</t>
+          <t xml:space="preserve">- 17: Gärtnerei / Gardening Shed (Spannenberg, bei (17,23)) nutzte fälschlich Bit 16 (wie Stadtgarten O) und nutzt jetzt 17. In der Binärdatei stand noch der alte Name Parkverwaltung.</t>
         </is>
       </c>
     </row>
     <row r="39" spans="1:1">
       <c r="A39" t="inlineStr">
         <is>
-          <t xml:space="preserve">- 101/102: Der Weise hatte in den Daten schon 101 statt wie geplant 102. Das Versteck hat jetzt 102. Bit 0 ist wie im Original unbenutzt, ab 107 ist alles frei.</t>
+          <t xml:space="preserve">- 101/102: Der Weise hatte in den Daten schon 101 statt wie geplant 102. Das Versteck hat jetzt 102 (Name im Spiel: Dunkles Haus, um nicht zu spoilern). Bit 0 ist wie im Original unbenutzt, ab 107 ist alles frei.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add the Bore quest: Bore joins after the forest moon and works in the mine of Dor Kiredon
- NPC Bore (24) in Gemstone is level 30. When leaving the forest moon he is replaced by the new
  party member 18 (dwarf warrior level 30), who tells about the forest moon, gives the first
  navstone, trades amber chunks for navstones and can join the party.
- Entering Dor Kiredon with Bore: he leaves the party with the remove party member event, his
  equipment and items go to the new extended chests 307/308 in the mine, he stays hidden in
  Gemstone, and the new NPC Bore (80) appears in the mine. Talking to him gives 5000 EXP once,
  then he trades navstones as well.
- Labdata 14 gets a chest object (block 61), new global vars 471/472.
- Texts in german and english (AllTexts), documented in the xlsx.
</commit_message>
<xml_diff>
--- a/AmbermoonAdvanced.xlsx
+++ b/AmbermoonAdvanced.xlsx
@@ -9955,7 +9955,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.28515625" customWidth="1"/>
@@ -10145,6 +10145,23 @@
         <v>1099</v>
       </c>
     </row>
+    <row r="13">
+      <c r="D13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">14</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mine Dor Kiredon (345)</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chest object (texture 164, like labdata 37) as block 61</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -10157,7 +10174,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="28.5703125" customWidth="1"/>
@@ -10453,6 +10470,74 @@
         <v>1125</v>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">343</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dor Kiredon</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chain 20 at (16,21) and (16,23): if Bore (18) is in the party, text 21, he leaves the party (chests 307/308), is hidden in Gemstone, the mine NPC and the chests appear, var 471 is set</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">345</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mine</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NPC Bore (80) at (12,7), chests 307/308 at (11,7) and (10,8) (only active with var 471, block 61 is placed by map 343)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">406</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gemstone Ruinen</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Party member Bore (18) at the position of NPC Bore, initially hidden</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">436</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">F-Schiff: Waldmond</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">When leaving the forest moon (var 320), NPC Bore is hidden and party member Bore is shown in Gemstone</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78749999999999998" bottom="0.78749999999999998" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -10461,7 +10546,7 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
-  <dimension ref="A1:O22"/>
+  <dimension ref="A1:O24"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="22" customWidth="1"/>
@@ -10780,6 +10865,50 @@
       </c>
       <c r="N22" t="s">
         <v>1180</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">80</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bore</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mine (345)</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bore after he left the party in Dor Kiredon. First talk gives 5000 EXP, trades amber chunks for navstones</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">24</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bore</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gemstone Ruinen (406)</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Now level 30. Hidden when leaving the forest moon (airship 436), replaced by party member 18</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -10793,7 +10922,7 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0E00-000000000000}">
-  <dimension ref="A1:H122"/>
+  <dimension ref="A1:H124"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.42578125" style="16" customWidth="1"/>
@@ -12263,6 +12392,40 @@
       </c>
       <c r="C122" t="s">
         <v>1407</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t xml:space="preserve">307 (X051)</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mine Dor Kiredon (345)</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bore's equipment (filled by the remove party member event)</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t xml:space="preserve">308 (X052)</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mine Dor Kiredon (345)</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bore's items (filled by the remove party member event)</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -12865,7 +13028,7 @@
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1200-000000000000}">
-  <dimension ref="A1:N27"/>
+  <dimension ref="A1:N28"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -13688,6 +13851,18 @@
       <c r="K27" s="32">
         <f>G7</f>
         <v>155</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bore</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">New party member 18: dwarf warrior level 30, 480 LP, 7 APR, helmet, war hammer, chain mail, dwarf shield, leather boots</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -21895,7 +22070,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:D253"/>
+  <dimension ref="A1:D255"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="63.42578125" customWidth="1"/>
@@ -23178,6 +23353,20 @@
     <row r="253" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A253" t="s">
         <v>384</v>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t xml:space="preserve">471: Bore left the party in Dor Kiredon and works in the mine (shows his 2 chests)</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t xml:space="preserve">472: Bore in the mine thanked the party (5000 EXP given)</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Song 33: temple version of Psychedelic Dune Groove in Music.amb, Max_music 33 in Set_music, Music sheet in the xlsx
</commit_message>
<xml_diff>
--- a/AmbermoonAdvanced.xlsx
+++ b/AmbermoonAdvanced.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Robert\source\repos\Ambermoon-Advanced\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01BE5FD5-D483-4664-8918-50ADC3B5FF44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD7A6C58-8889-41D9-9BA5-C3AB2CE4F5CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" firstSheet="6" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" firstSheet="36" activeTab="42" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Neue Daten Ep3" sheetId="1" r:id="rId1"/>
@@ -55,6 +55,7 @@
     <sheet name="CombatBackgrounds" sheetId="40" r:id="rId40"/>
     <sheet name="ElementChanges" sheetId="41" r:id="rId41"/>
     <sheet name="Shards" sheetId="42" r:id="rId42"/>
+    <sheet name="Music" sheetId="43" r:id="rId43"/>
   </sheets>
   <calcPr calcId="191029" iterate="1" iterateDelta="1E-4"/>
   <extLst>
@@ -77,7 +78,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3101" uniqueCount="2217">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3176" uniqueCount="2285">
   <si>
     <t>Map texts</t>
   </si>
@@ -6845,6 +6846,210 @@
   </si>
   <si>
     <t>Flag 12 (no travel music) set, map music 2 (Mellow Camel Funk)</t>
+  </si>
+  <si>
+    <t>Original usage</t>
+  </si>
+  <si>
+    <t>Advanced usage</t>
+  </si>
+  <si>
+    <t>Who Said Hi Ho</t>
+  </si>
+  <si>
+    <t>Gnome mine</t>
+  </si>
+  <si>
+    <t>Mellow Camel Funk</t>
+  </si>
+  <si>
+    <t>Morag places and sand lizard (riding)</t>
+  </si>
+  <si>
+    <t>Morag world maps 513-528 (map flag 12: no travel music)</t>
+  </si>
+  <si>
+    <t>Close To The Hedge</t>
+  </si>
+  <si>
+    <t>Dwarfs, forest moon indoor</t>
+  </si>
+  <si>
+    <t>Voice Of The Bagpipe</t>
+  </si>
+  <si>
+    <t>Gemstone</t>
+  </si>
+  <si>
+    <t>Downtown</t>
+  </si>
+  <si>
+    <t>Ship</t>
+  </si>
+  <si>
+    <t>Ship (sailing)</t>
+  </si>
+  <si>
+    <t>Whole Lotta Dove</t>
+  </si>
+  <si>
+    <t>Eagle (flying)</t>
+  </si>
+  <si>
+    <t>Horse Is No Disgrace</t>
+  </si>
+  <si>
+    <t>Horse (riding)</t>
+  </si>
+  <si>
+    <t>Don't Look Bach</t>
+  </si>
+  <si>
+    <t>Taverns</t>
+  </si>
+  <si>
+    <t>Rough Waterfront Tavern</t>
+  </si>
+  <si>
+    <t>Sapphire Fireballs Of Pure Love</t>
+  </si>
+  <si>
+    <t>Battle theme</t>
+  </si>
+  <si>
+    <t>The Aum Remains The Same</t>
+  </si>
+  <si>
+    <t>Temple of life</t>
+  </si>
+  <si>
+    <t>Capital</t>
+  </si>
+  <si>
+    <t>Newlake</t>
+  </si>
+  <si>
+    <t>Plodding Along</t>
+  </si>
+  <si>
+    <t>All world maps</t>
+  </si>
+  <si>
+    <t>Compact Disc</t>
+  </si>
+  <si>
+    <t>Magical fly disc</t>
+  </si>
+  <si>
+    <t>Riverside Travelling Blues</t>
+  </si>
+  <si>
+    <t>Nobodys Vault But Mine</t>
+  </si>
+  <si>
+    <t>Thief guild</t>
+  </si>
+  <si>
+    <t>La Crypta Strangiato</t>
+  </si>
+  <si>
+    <t>Grandfather's cellar</t>
+  </si>
+  <si>
+    <t>Misty Dungeon Hop</t>
+  </si>
+  <si>
+    <t>Alchemist tower</t>
+  </si>
+  <si>
+    <t>Burn Baby Burn</t>
+  </si>
+  <si>
+    <t>Witch's broom, Nera's house</t>
+  </si>
+  <si>
+    <t>Bar Brawlin</t>
+  </si>
+  <si>
+    <t>Camp, Inn</t>
+  </si>
+  <si>
+    <t>Psychedelic Dune Groove</t>
+  </si>
+  <si>
+    <t>Sand ship</t>
+  </si>
+  <si>
+    <t>Base of song 33</t>
+  </si>
+  <si>
+    <t>Stairway To Level 50</t>
+  </si>
+  <si>
+    <t>Level up</t>
+  </si>
+  <si>
+    <t>That Hunch Is Back</t>
+  </si>
+  <si>
+    <t>Undeads</t>
+  </si>
+  <si>
+    <t>ChickenSoup</t>
+  </si>
+  <si>
+    <t>Superman mode, Thalion office</t>
+  </si>
+  <si>
+    <t>Dragon Chase In Creepy Dungeon</t>
+  </si>
+  <si>
+    <t>Luminor's tower</t>
+  </si>
+  <si>
+    <t>His Masters Voice</t>
+  </si>
+  <si>
+    <t>Harp, Matthias in Illien</t>
+  </si>
+  <si>
+    <t>No Name</t>
+  </si>
+  <si>
+    <t>House of healers</t>
+  </si>
+  <si>
+    <t>Oh No Not Another Magical Event</t>
+  </si>
+  <si>
+    <t>Magical events (wishing well, pulsing lights, etc)</t>
+  </si>
+  <si>
+    <t>The Uh Oh Song</t>
+  </si>
+  <si>
+    <t>Dramatic events</t>
+  </si>
+  <si>
+    <t>Owner Of A Lonely Sword</t>
+  </si>
+  <si>
+    <t>Grandfather's house</t>
+  </si>
+  <si>
+    <t>Game Over</t>
+  </si>
+  <si>
+    <t>Psychedelic Dune Groove (Temple)</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>Council temple (which one: open)</t>
+  </si>
+  <si>
+    <t>New in Advanced. Song 22 starting and looping at position 34, positions 52-53 and the last 3 removed (about 60 s per loop). Source: assets/Temples/music/SONIC.PsychedelicDuneGroove_ab34_cut2. Code: Max_music = 33 in Set_music (the harp still shows 32 songs). Remake support missing.</t>
   </si>
 </sst>
 </file>
@@ -7490,17 +7695,17 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="21" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="27" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="27" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="21" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -16888,14 +17093,14 @@
       <c r="B32" s="54" t="s">
         <v>1745</v>
       </c>
-      <c r="C32" s="78" t="s">
+      <c r="C32" s="75" t="s">
         <v>1746</v>
       </c>
-      <c r="D32" s="78"/>
-      <c r="E32" s="78"/>
-      <c r="F32" s="78"/>
-      <c r="G32" s="78"/>
-      <c r="H32" s="78"/>
+      <c r="D32" s="75"/>
+      <c r="E32" s="75"/>
+      <c r="F32" s="75"/>
+      <c r="G32" s="75"/>
+      <c r="H32" s="75"/>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" s="36" t="s">
@@ -16904,14 +17109,14 @@
       <c r="B33" s="28" t="s">
         <v>1748</v>
       </c>
-      <c r="C33" s="77" t="s">
+      <c r="C33" s="76" t="s">
         <v>1749</v>
       </c>
-      <c r="D33" s="77"/>
-      <c r="E33" s="77"/>
-      <c r="F33" s="77"/>
-      <c r="G33" s="77"/>
-      <c r="H33" s="77"/>
+      <c r="D33" s="76"/>
+      <c r="E33" s="76"/>
+      <c r="F33" s="76"/>
+      <c r="G33" s="76"/>
+      <c r="H33" s="76"/>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" s="36" t="s">
@@ -16920,14 +17125,14 @@
       <c r="B34" s="28" t="s">
         <v>1748</v>
       </c>
-      <c r="C34" s="77" t="s">
+      <c r="C34" s="76" t="s">
         <v>1749</v>
       </c>
-      <c r="D34" s="77"/>
-      <c r="E34" s="77"/>
-      <c r="F34" s="77"/>
-      <c r="G34" s="77"/>
-      <c r="H34" s="77"/>
+      <c r="D34" s="76"/>
+      <c r="E34" s="76"/>
+      <c r="F34" s="76"/>
+      <c r="G34" s="76"/>
+      <c r="H34" s="76"/>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" s="36" t="s">
@@ -16936,14 +17141,14 @@
       <c r="B35" s="28" t="s">
         <v>1748</v>
       </c>
-      <c r="C35" s="77" t="s">
+      <c r="C35" s="76" t="s">
         <v>1749</v>
       </c>
-      <c r="D35" s="77"/>
-      <c r="E35" s="77"/>
-      <c r="F35" s="77"/>
-      <c r="G35" s="77"/>
-      <c r="H35" s="77"/>
+      <c r="D35" s="76"/>
+      <c r="E35" s="76"/>
+      <c r="F35" s="76"/>
+      <c r="G35" s="76"/>
+      <c r="H35" s="76"/>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" s="36" t="s">
@@ -16952,14 +17157,14 @@
       <c r="B36" s="28" t="s">
         <v>1734</v>
       </c>
-      <c r="C36" s="76" t="s">
+      <c r="C36" s="77" t="s">
         <v>1753</v>
       </c>
-      <c r="D36" s="76"/>
-      <c r="E36" s="76"/>
-      <c r="F36" s="76"/>
-      <c r="G36" s="76"/>
-      <c r="H36" s="76"/>
+      <c r="D36" s="77"/>
+      <c r="E36" s="77"/>
+      <c r="F36" s="77"/>
+      <c r="G36" s="77"/>
+      <c r="H36" s="77"/>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" s="36" t="s">
@@ -16968,14 +17173,14 @@
       <c r="B37" s="28" t="s">
         <v>1736</v>
       </c>
-      <c r="C37" s="77" t="s">
+      <c r="C37" s="76" t="s">
         <v>1755</v>
       </c>
-      <c r="D37" s="77"/>
-      <c r="E37" s="77"/>
-      <c r="F37" s="77"/>
-      <c r="G37" s="77"/>
-      <c r="H37" s="77"/>
+      <c r="D37" s="76"/>
+      <c r="E37" s="76"/>
+      <c r="F37" s="76"/>
+      <c r="G37" s="76"/>
+      <c r="H37" s="76"/>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" s="36" t="s">
@@ -16984,14 +17189,14 @@
       <c r="B38" s="28" t="s">
         <v>1734</v>
       </c>
-      <c r="C38" s="77" t="s">
+      <c r="C38" s="76" t="s">
         <v>1755</v>
       </c>
-      <c r="D38" s="77"/>
-      <c r="E38" s="77"/>
-      <c r="F38" s="77"/>
-      <c r="G38" s="77"/>
-      <c r="H38" s="77"/>
+      <c r="D38" s="76"/>
+      <c r="E38" s="76"/>
+      <c r="F38" s="76"/>
+      <c r="G38" s="76"/>
+      <c r="H38" s="76"/>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" s="36" t="s">
@@ -17000,14 +17205,14 @@
       <c r="B39" s="28" t="s">
         <v>1734</v>
       </c>
-      <c r="C39" s="76" t="s">
+      <c r="C39" s="77" t="s">
         <v>1753</v>
       </c>
-      <c r="D39" s="76"/>
-      <c r="E39" s="76"/>
-      <c r="F39" s="76"/>
-      <c r="G39" s="76"/>
-      <c r="H39" s="76"/>
+      <c r="D39" s="77"/>
+      <c r="E39" s="77"/>
+      <c r="F39" s="77"/>
+      <c r="G39" s="77"/>
+      <c r="H39" s="77"/>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" s="36" t="s">
@@ -17016,14 +17221,14 @@
       <c r="B40" s="28" t="s">
         <v>1734</v>
       </c>
-      <c r="C40" s="76" t="s">
+      <c r="C40" s="77" t="s">
         <v>1753</v>
       </c>
-      <c r="D40" s="76"/>
-      <c r="E40" s="76"/>
-      <c r="F40" s="76"/>
-      <c r="G40" s="76"/>
-      <c r="H40" s="76"/>
+      <c r="D40" s="77"/>
+      <c r="E40" s="77"/>
+      <c r="F40" s="77"/>
+      <c r="G40" s="77"/>
+      <c r="H40" s="77"/>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" s="36" t="s">
@@ -17032,14 +17237,14 @@
       <c r="B41" s="28" t="s">
         <v>1737</v>
       </c>
-      <c r="C41" s="76" t="s">
+      <c r="C41" s="77" t="s">
         <v>1759</v>
       </c>
-      <c r="D41" s="76"/>
-      <c r="E41" s="76"/>
-      <c r="F41" s="76"/>
-      <c r="G41" s="76"/>
-      <c r="H41" s="76"/>
+      <c r="D41" s="77"/>
+      <c r="E41" s="77"/>
+      <c r="F41" s="77"/>
+      <c r="G41" s="77"/>
+      <c r="H41" s="77"/>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" s="36" t="s">
@@ -17048,14 +17253,14 @@
       <c r="B42" s="28" t="s">
         <v>1738</v>
       </c>
-      <c r="C42" s="76" t="s">
+      <c r="C42" s="77" t="s">
         <v>1761</v>
       </c>
-      <c r="D42" s="76"/>
-      <c r="E42" s="76"/>
-      <c r="F42" s="76"/>
-      <c r="G42" s="76"/>
-      <c r="H42" s="76"/>
+      <c r="D42" s="77"/>
+      <c r="E42" s="77"/>
+      <c r="F42" s="77"/>
+      <c r="G42" s="77"/>
+      <c r="H42" s="77"/>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" s="36" t="s">
@@ -17064,14 +17269,14 @@
       <c r="B43" s="28" t="s">
         <v>1739</v>
       </c>
-      <c r="C43" s="76" t="s">
+      <c r="C43" s="77" t="s">
         <v>1763</v>
       </c>
-      <c r="D43" s="76"/>
-      <c r="E43" s="76"/>
-      <c r="F43" s="76"/>
-      <c r="G43" s="76"/>
-      <c r="H43" s="76"/>
+      <c r="D43" s="77"/>
+      <c r="E43" s="77"/>
+      <c r="F43" s="77"/>
+      <c r="G43" s="77"/>
+      <c r="H43" s="77"/>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" s="36" t="s">
@@ -17080,26 +17285,26 @@
       <c r="B44" s="28" t="s">
         <v>1740</v>
       </c>
-      <c r="C44" s="76" t="s">
+      <c r="C44" s="77" t="s">
         <v>1765</v>
       </c>
-      <c r="D44" s="76"/>
-      <c r="E44" s="76"/>
-      <c r="F44" s="76"/>
-      <c r="G44" s="76"/>
-      <c r="H44" s="76"/>
+      <c r="D44" s="77"/>
+      <c r="E44" s="77"/>
+      <c r="F44" s="77"/>
+      <c r="G44" s="77"/>
+      <c r="H44" s="77"/>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A48" s="75" t="s">
+      <c r="A48" s="78" t="s">
         <v>1754</v>
       </c>
-      <c r="B48" s="75"/>
-      <c r="C48" s="75"/>
-      <c r="D48" s="75"/>
-      <c r="E48" s="75"/>
-      <c r="F48" s="75"/>
-      <c r="G48" s="75"/>
-      <c r="H48" s="75"/>
+      <c r="B48" s="78"/>
+      <c r="C48" s="78"/>
+      <c r="D48" s="78"/>
+      <c r="E48" s="78"/>
+      <c r="F48" s="78"/>
+      <c r="G48" s="78"/>
+      <c r="H48" s="78"/>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
@@ -17112,16 +17317,16 @@
       </c>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A52" s="75" t="s">
+      <c r="A52" s="78" t="s">
         <v>1756</v>
       </c>
-      <c r="B52" s="75"/>
-      <c r="C52" s="75"/>
-      <c r="D52" s="75"/>
-      <c r="E52" s="75"/>
-      <c r="F52" s="75"/>
-      <c r="G52" s="75"/>
-      <c r="H52" s="75"/>
+      <c r="B52" s="78"/>
+      <c r="C52" s="78"/>
+      <c r="D52" s="78"/>
+      <c r="E52" s="78"/>
+      <c r="F52" s="78"/>
+      <c r="G52" s="78"/>
+      <c r="H52" s="78"/>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
@@ -17129,16 +17334,16 @@
       </c>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A57" s="75" t="s">
+      <c r="A57" s="78" t="s">
         <v>1769</v>
       </c>
-      <c r="B57" s="75"/>
-      <c r="C57" s="75"/>
-      <c r="D57" s="75"/>
-      <c r="E57" s="75"/>
-      <c r="F57" s="75"/>
-      <c r="G57" s="75"/>
-      <c r="H57" s="75"/>
+      <c r="B57" s="78"/>
+      <c r="C57" s="78"/>
+      <c r="D57" s="78"/>
+      <c r="E57" s="78"/>
+      <c r="F57" s="78"/>
+      <c r="G57" s="78"/>
+      <c r="H57" s="78"/>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
@@ -17206,12 +17411,12 @@
       </c>
     </row>
     <row r="73" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="H73" s="75" t="s">
+      <c r="H73" s="78" t="s">
         <v>1783</v>
       </c>
-      <c r="I73" s="75"/>
-      <c r="J73" s="75"/>
-      <c r="K73" s="75"/>
+      <c r="I73" s="78"/>
+      <c r="J73" s="78"/>
+      <c r="K73" s="78"/>
     </row>
     <row r="74" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A74" s="55" t="s">
@@ -17778,16 +17983,6 @@
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="C32:H32"/>
-    <mergeCell ref="C33:H33"/>
-    <mergeCell ref="C34:H34"/>
-    <mergeCell ref="C35:H35"/>
-    <mergeCell ref="C36:H36"/>
-    <mergeCell ref="C37:H37"/>
-    <mergeCell ref="C38:H38"/>
-    <mergeCell ref="C39:H39"/>
-    <mergeCell ref="C40:H40"/>
-    <mergeCell ref="C41:H41"/>
     <mergeCell ref="A57:H57"/>
     <mergeCell ref="H73:K73"/>
     <mergeCell ref="C42:H42"/>
@@ -17795,6 +17990,16 @@
     <mergeCell ref="C44:H44"/>
     <mergeCell ref="A48:H48"/>
     <mergeCell ref="A52:H52"/>
+    <mergeCell ref="C37:H37"/>
+    <mergeCell ref="C38:H38"/>
+    <mergeCell ref="C39:H39"/>
+    <mergeCell ref="C40:H40"/>
+    <mergeCell ref="C41:H41"/>
+    <mergeCell ref="C32:H32"/>
+    <mergeCell ref="C33:H33"/>
+    <mergeCell ref="C34:H34"/>
+    <mergeCell ref="C35:H35"/>
+    <mergeCell ref="C36:H36"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78749999999999998" bottom="0.78749999999999998" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -17857,13 +18062,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="75" t="s">
+      <c r="A1" s="78" t="s">
         <v>1905</v>
       </c>
-      <c r="B1" s="75"/>
-      <c r="C1" s="75"/>
-      <c r="D1" s="75"/>
-      <c r="E1" s="75"/>
+      <c r="B1" s="78"/>
+      <c r="C1" s="78"/>
+      <c r="D1" s="78"/>
+      <c r="E1" s="78"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="56" t="s">
@@ -21799,6 +22004,415 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9EB917A5-DF3B-4EE0-9368-5DECBA5FA2AE}">
+  <dimension ref="A1:E34"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="6" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="32.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="44.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="51.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="255.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" s="67" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="67" t="s">
+        <v>397</v>
+      </c>
+      <c r="B1" s="67" t="s">
+        <v>398</v>
+      </c>
+      <c r="C1" s="67" t="s">
+        <v>2217</v>
+      </c>
+      <c r="D1" s="67" t="s">
+        <v>2218</v>
+      </c>
+      <c r="E1" s="67" t="s">
+        <v>1746</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>2219</v>
+      </c>
+      <c r="C2" t="s">
+        <v>2220</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>2221</v>
+      </c>
+      <c r="C3" t="s">
+        <v>2222</v>
+      </c>
+      <c r="D3" t="s">
+        <v>2223</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>2224</v>
+      </c>
+      <c r="C4" t="s">
+        <v>2225</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>2226</v>
+      </c>
+      <c r="C5" t="s">
+        <v>2227</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>2228</v>
+      </c>
+      <c r="C6" t="s">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>2229</v>
+      </c>
+      <c r="C7" t="s">
+        <v>2230</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>2231</v>
+      </c>
+      <c r="C8" t="s">
+        <v>2232</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>2233</v>
+      </c>
+      <c r="C9" t="s">
+        <v>2234</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>2235</v>
+      </c>
+      <c r="C10" t="s">
+        <v>2236</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>2237</v>
+      </c>
+      <c r="C11" t="s">
+        <v>2236</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>2238</v>
+      </c>
+      <c r="C12" t="s">
+        <v>2239</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>2240</v>
+      </c>
+      <c r="C13" t="s">
+        <v>2241</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
+        <v>2242</v>
+      </c>
+      <c r="C14" t="s">
+        <v>2243</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>2244</v>
+      </c>
+      <c r="C15" t="s">
+        <v>2245</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="s">
+        <v>2246</v>
+      </c>
+      <c r="C16" t="s">
+        <v>2247</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="s">
+        <v>2248</v>
+      </c>
+      <c r="C17" t="s">
+        <v>493</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" t="s">
+        <v>2249</v>
+      </c>
+      <c r="C18" t="s">
+        <v>2250</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" t="s">
+        <v>2251</v>
+      </c>
+      <c r="C19" t="s">
+        <v>2252</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" t="s">
+        <v>2253</v>
+      </c>
+      <c r="C20" t="s">
+        <v>2254</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21" t="s">
+        <v>2255</v>
+      </c>
+      <c r="C21" t="s">
+        <v>2256</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22" t="s">
+        <v>2257</v>
+      </c>
+      <c r="C22" t="s">
+        <v>2258</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23" t="s">
+        <v>2259</v>
+      </c>
+      <c r="C23" t="s">
+        <v>2260</v>
+      </c>
+      <c r="E23" t="s">
+        <v>2261</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24" t="s">
+        <v>2262</v>
+      </c>
+      <c r="C24" t="s">
+        <v>2263</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25" t="s">
+        <v>2264</v>
+      </c>
+      <c r="C25" t="s">
+        <v>2265</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26" t="s">
+        <v>2266</v>
+      </c>
+      <c r="C26" t="s">
+        <v>2267</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>26</v>
+      </c>
+      <c r="B27" t="s">
+        <v>2268</v>
+      </c>
+      <c r="C27" t="s">
+        <v>2269</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A28">
+        <v>27</v>
+      </c>
+      <c r="B28" t="s">
+        <v>2270</v>
+      </c>
+      <c r="C28" t="s">
+        <v>2271</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A29">
+        <v>28</v>
+      </c>
+      <c r="B29" t="s">
+        <v>2272</v>
+      </c>
+      <c r="C29" t="s">
+        <v>2273</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A30">
+        <v>29</v>
+      </c>
+      <c r="B30" t="s">
+        <v>2274</v>
+      </c>
+      <c r="C30" t="s">
+        <v>2275</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A31">
+        <v>30</v>
+      </c>
+      <c r="B31" t="s">
+        <v>2276</v>
+      </c>
+      <c r="C31" t="s">
+        <v>2277</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A32">
+        <v>31</v>
+      </c>
+      <c r="B32" t="s">
+        <v>2278</v>
+      </c>
+      <c r="C32" t="s">
+        <v>2279</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A33">
+        <v>32</v>
+      </c>
+      <c r="B33" t="s">
+        <v>2280</v>
+      </c>
+      <c r="C33" t="s">
+        <v>2280</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A34">
+        <v>33</v>
+      </c>
+      <c r="B34" t="s">
+        <v>2281</v>
+      </c>
+      <c r="C34" t="s">
+        <v>2282</v>
+      </c>
+      <c r="D34" t="s">
+        <v>2283</v>
+      </c>
+      <c r="E34" t="s">
+        <v>2284</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:D255"/>

</xml_diff>

<commit_message>
Temple prototype S'Riel (map 487): labdata 46, palette 59, texts DE/EN, automaps 485-487 in Save.00
</commit_message>
<xml_diff>
--- a/AmbermoonAdvanced.xlsx
+++ b/AmbermoonAdvanced.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Robert\source\repos\Ambermoon-Advanced\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD7A6C58-8889-41D9-9BA5-C3AB2CE4F5CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{715E6CB1-654C-47A9-B89E-A0331E10411F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" firstSheet="36" activeTab="42" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -78,7 +78,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3176" uniqueCount="2285">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3181" uniqueCount="2289">
   <si>
     <t>Map texts</t>
   </si>
@@ -7046,10 +7046,22 @@
     <t>-</t>
   </si>
   <si>
-    <t>Council temple (which one: open)</t>
-  </si>
-  <si>
     <t>New in Advanced. Song 22 starting and looping at position 34, positions 52-53 and the last 3 removed (about 60 s per loop). Source: assets/Temples/music/SONIC.PsychedelicDuneGroove_ab34_cut2. Code: Max_music = 33 in Set_music (the harp still shows 32 songs). Remake support missing.</t>
+  </si>
+  <si>
+    <t>Palast des S'Riel (Prototyp) / Palace of S'Riel (prototype)</t>
+  </si>
+  <si>
+    <t>Temple rework pilot, only reachable with the cheat map jump (t, 487). Built by assets/Temples/tools/build_prototype.py. Labdata 46, palette 59, music 33. Exit to 520 (37,41) like 444. Reuses chests 116/117 of map 444.</t>
+  </si>
+  <si>
+    <t>S'Riel prototype (487): copy of labdata 5 (Gala temple) with floor 20 and ceiling 8. Palette 59 (Sandstein) is new too.</t>
+  </si>
+  <si>
+    <t>Add automaps 485 (27x27, 92 bytes), 486 (11x19, 27 bytes) and 487 (17x17, 37 bytes). They were missing in Save.00, entering 485/486 on the Amiga ends in a fatal error (Init_automap loads the entry for every 3D map).</t>
+  </si>
+  <si>
+    <t>Prototype map 487 (S'Riel); final temple open</t>
   </si>
 </sst>
 </file>
@@ -7674,14 +7686,14 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -7695,17 +7707,17 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="27" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="21" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="27" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="21" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -7918,22 +7930,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A1" s="69" t="s">
+      <c r="A1" s="68" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="69"/>
-      <c r="E1" s="69" t="s">
+      <c r="B1" s="68"/>
+      <c r="E1" s="68" t="s">
         <v>1</v>
       </c>
-      <c r="F1" s="69"/>
-      <c r="I1" s="69" t="s">
+      <c r="F1" s="68"/>
+      <c r="I1" s="68" t="s">
         <v>2</v>
       </c>
-      <c r="J1" s="69"/>
-      <c r="M1" s="69" t="s">
+      <c r="J1" s="68"/>
+      <c r="M1" s="68" t="s">
         <v>3</v>
       </c>
-      <c r="N1" s="69"/>
+      <c r="N1" s="68"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2">
@@ -8018,26 +8030,26 @@
       </c>
     </row>
     <row r="21" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A21" s="69" t="s">
+      <c r="A21" s="68" t="s">
         <v>11</v>
       </c>
-      <c r="B21" s="69"/>
-      <c r="E21" s="69" t="s">
+      <c r="B21" s="68"/>
+      <c r="E21" s="68" t="s">
         <v>12</v>
       </c>
-      <c r="F21" s="69"/>
-      <c r="I21" s="69" t="s">
+      <c r="F21" s="68"/>
+      <c r="I21" s="68" t="s">
         <v>13</v>
       </c>
-      <c r="J21" s="69"/>
-      <c r="M21" s="69" t="s">
+      <c r="J21" s="68"/>
+      <c r="M21" s="68" t="s">
         <v>14</v>
       </c>
-      <c r="N21" s="69"/>
-      <c r="Q21" s="69" t="s">
+      <c r="N21" s="68"/>
+      <c r="Q21" s="68" t="s">
         <v>15</v>
       </c>
-      <c r="R21" s="69"/>
+      <c r="R21" s="68"/>
     </row>
     <row r="22" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A22">
@@ -9300,7 +9312,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
-  <dimension ref="A1:D47"/>
+  <dimension ref="A1:D48"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7.7109375" customWidth="1"/>
@@ -9936,6 +9948,20 @@
         <v>986</v>
       </c>
     </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A48">
+        <v>487</v>
+      </c>
+      <c r="B48" t="s">
+        <v>2284</v>
+      </c>
+      <c r="C48" t="s">
+        <v>911</v>
+      </c>
+      <c r="D48" t="s">
+        <v>2285</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78749999999999998" bottom="0.78749999999999998" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -9944,7 +9970,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.28515625" customWidth="1"/>
@@ -10143,6 +10169,14 @@
       </c>
       <c r="F13" t="s">
         <v>2193</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>46</v>
+      </c>
+      <c r="B14" t="s">
+        <v>2286</v>
       </c>
     </row>
   </sheetData>
@@ -10896,10 +10930,10 @@
       <c r="C1" t="s">
         <v>1100</v>
       </c>
-      <c r="E1" s="68" t="s">
+      <c r="E1" s="70" t="s">
         <v>1101</v>
       </c>
-      <c r="F1" s="68"/>
+      <c r="F1" s="70"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="16">
@@ -11137,10 +11171,10 @@
       <c r="C16" t="s">
         <v>1132</v>
       </c>
-      <c r="E16" s="68" t="s">
+      <c r="E16" s="70" t="s">
         <v>1133</v>
       </c>
-      <c r="F16" s="68"/>
+      <c r="F16" s="70"/>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="16">
@@ -11220,10 +11254,10 @@
       <c r="C21" t="s">
         <v>1143</v>
       </c>
-      <c r="E21" s="68" t="s">
+      <c r="E21" s="70" t="s">
         <v>1144</v>
       </c>
-      <c r="F21" s="68"/>
+      <c r="F21" s="70"/>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" s="16">
@@ -15982,16 +16016,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" s="68" t="s">
+      <c r="A1" s="70" t="s">
         <v>1617</v>
       </c>
-      <c r="B1" s="68"/>
-      <c r="C1" s="68"/>
-      <c r="G1" s="68" t="s">
+      <c r="B1" s="70"/>
+      <c r="C1" s="70"/>
+      <c r="G1" s="70" t="s">
         <v>1618</v>
       </c>
-      <c r="H1" s="68"/>
-      <c r="I1" s="68"/>
+      <c r="H1" s="70"/>
+      <c r="I1" s="70"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
@@ -16199,17 +16233,17 @@
       <c r="A1" s="43" t="s">
         <v>1621</v>
       </c>
-      <c r="C1" s="68" t="s">
+      <c r="C1" s="70" t="s">
         <v>1622</v>
       </c>
-      <c r="D1" s="68"/>
-      <c r="E1" s="68"/>
-      <c r="G1" s="68" t="s">
+      <c r="D1" s="70"/>
+      <c r="E1" s="70"/>
+      <c r="G1" s="70" t="s">
         <v>1623</v>
       </c>
-      <c r="H1" s="68"/>
-      <c r="I1" s="68"/>
-      <c r="J1" s="68"/>
+      <c r="H1" s="70"/>
+      <c r="I1" s="70"/>
+      <c r="J1" s="70"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
@@ -17093,14 +17127,14 @@
       <c r="B32" s="54" t="s">
         <v>1745</v>
       </c>
-      <c r="C32" s="75" t="s">
+      <c r="C32" s="78" t="s">
         <v>1746</v>
       </c>
-      <c r="D32" s="75"/>
-      <c r="E32" s="75"/>
-      <c r="F32" s="75"/>
-      <c r="G32" s="75"/>
-      <c r="H32" s="75"/>
+      <c r="D32" s="78"/>
+      <c r="E32" s="78"/>
+      <c r="F32" s="78"/>
+      <c r="G32" s="78"/>
+      <c r="H32" s="78"/>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" s="36" t="s">
@@ -17109,14 +17143,14 @@
       <c r="B33" s="28" t="s">
         <v>1748</v>
       </c>
-      <c r="C33" s="76" t="s">
+      <c r="C33" s="77" t="s">
         <v>1749</v>
       </c>
-      <c r="D33" s="76"/>
-      <c r="E33" s="76"/>
-      <c r="F33" s="76"/>
-      <c r="G33" s="76"/>
-      <c r="H33" s="76"/>
+      <c r="D33" s="77"/>
+      <c r="E33" s="77"/>
+      <c r="F33" s="77"/>
+      <c r="G33" s="77"/>
+      <c r="H33" s="77"/>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" s="36" t="s">
@@ -17125,14 +17159,14 @@
       <c r="B34" s="28" t="s">
         <v>1748</v>
       </c>
-      <c r="C34" s="76" t="s">
+      <c r="C34" s="77" t="s">
         <v>1749</v>
       </c>
-      <c r="D34" s="76"/>
-      <c r="E34" s="76"/>
-      <c r="F34" s="76"/>
-      <c r="G34" s="76"/>
-      <c r="H34" s="76"/>
+      <c r="D34" s="77"/>
+      <c r="E34" s="77"/>
+      <c r="F34" s="77"/>
+      <c r="G34" s="77"/>
+      <c r="H34" s="77"/>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" s="36" t="s">
@@ -17141,14 +17175,14 @@
       <c r="B35" s="28" t="s">
         <v>1748</v>
       </c>
-      <c r="C35" s="76" t="s">
+      <c r="C35" s="77" t="s">
         <v>1749</v>
       </c>
-      <c r="D35" s="76"/>
-      <c r="E35" s="76"/>
-      <c r="F35" s="76"/>
-      <c r="G35" s="76"/>
-      <c r="H35" s="76"/>
+      <c r="D35" s="77"/>
+      <c r="E35" s="77"/>
+      <c r="F35" s="77"/>
+      <c r="G35" s="77"/>
+      <c r="H35" s="77"/>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" s="36" t="s">
@@ -17157,14 +17191,14 @@
       <c r="B36" s="28" t="s">
         <v>1734</v>
       </c>
-      <c r="C36" s="77" t="s">
+      <c r="C36" s="76" t="s">
         <v>1753</v>
       </c>
-      <c r="D36" s="77"/>
-      <c r="E36" s="77"/>
-      <c r="F36" s="77"/>
-      <c r="G36" s="77"/>
-      <c r="H36" s="77"/>
+      <c r="D36" s="76"/>
+      <c r="E36" s="76"/>
+      <c r="F36" s="76"/>
+      <c r="G36" s="76"/>
+      <c r="H36" s="76"/>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" s="36" t="s">
@@ -17173,14 +17207,14 @@
       <c r="B37" s="28" t="s">
         <v>1736</v>
       </c>
-      <c r="C37" s="76" t="s">
+      <c r="C37" s="77" t="s">
         <v>1755</v>
       </c>
-      <c r="D37" s="76"/>
-      <c r="E37" s="76"/>
-      <c r="F37" s="76"/>
-      <c r="G37" s="76"/>
-      <c r="H37" s="76"/>
+      <c r="D37" s="77"/>
+      <c r="E37" s="77"/>
+      <c r="F37" s="77"/>
+      <c r="G37" s="77"/>
+      <c r="H37" s="77"/>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" s="36" t="s">
@@ -17189,14 +17223,14 @@
       <c r="B38" s="28" t="s">
         <v>1734</v>
       </c>
-      <c r="C38" s="76" t="s">
+      <c r="C38" s="77" t="s">
         <v>1755</v>
       </c>
-      <c r="D38" s="76"/>
-      <c r="E38" s="76"/>
-      <c r="F38" s="76"/>
-      <c r="G38" s="76"/>
-      <c r="H38" s="76"/>
+      <c r="D38" s="77"/>
+      <c r="E38" s="77"/>
+      <c r="F38" s="77"/>
+      <c r="G38" s="77"/>
+      <c r="H38" s="77"/>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" s="36" t="s">
@@ -17205,14 +17239,14 @@
       <c r="B39" s="28" t="s">
         <v>1734</v>
       </c>
-      <c r="C39" s="77" t="s">
+      <c r="C39" s="76" t="s">
         <v>1753</v>
       </c>
-      <c r="D39" s="77"/>
-      <c r="E39" s="77"/>
-      <c r="F39" s="77"/>
-      <c r="G39" s="77"/>
-      <c r="H39" s="77"/>
+      <c r="D39" s="76"/>
+      <c r="E39" s="76"/>
+      <c r="F39" s="76"/>
+      <c r="G39" s="76"/>
+      <c r="H39" s="76"/>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" s="36" t="s">
@@ -17221,14 +17255,14 @@
       <c r="B40" s="28" t="s">
         <v>1734</v>
       </c>
-      <c r="C40" s="77" t="s">
+      <c r="C40" s="76" t="s">
         <v>1753</v>
       </c>
-      <c r="D40" s="77"/>
-      <c r="E40" s="77"/>
-      <c r="F40" s="77"/>
-      <c r="G40" s="77"/>
-      <c r="H40" s="77"/>
+      <c r="D40" s="76"/>
+      <c r="E40" s="76"/>
+      <c r="F40" s="76"/>
+      <c r="G40" s="76"/>
+      <c r="H40" s="76"/>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" s="36" t="s">
@@ -17237,14 +17271,14 @@
       <c r="B41" s="28" t="s">
         <v>1737</v>
       </c>
-      <c r="C41" s="77" t="s">
+      <c r="C41" s="76" t="s">
         <v>1759</v>
       </c>
-      <c r="D41" s="77"/>
-      <c r="E41" s="77"/>
-      <c r="F41" s="77"/>
-      <c r="G41" s="77"/>
-      <c r="H41" s="77"/>
+      <c r="D41" s="76"/>
+      <c r="E41" s="76"/>
+      <c r="F41" s="76"/>
+      <c r="G41" s="76"/>
+      <c r="H41" s="76"/>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" s="36" t="s">
@@ -17253,14 +17287,14 @@
       <c r="B42" s="28" t="s">
         <v>1738</v>
       </c>
-      <c r="C42" s="77" t="s">
+      <c r="C42" s="76" t="s">
         <v>1761</v>
       </c>
-      <c r="D42" s="77"/>
-      <c r="E42" s="77"/>
-      <c r="F42" s="77"/>
-      <c r="G42" s="77"/>
-      <c r="H42" s="77"/>
+      <c r="D42" s="76"/>
+      <c r="E42" s="76"/>
+      <c r="F42" s="76"/>
+      <c r="G42" s="76"/>
+      <c r="H42" s="76"/>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" s="36" t="s">
@@ -17269,14 +17303,14 @@
       <c r="B43" s="28" t="s">
         <v>1739</v>
       </c>
-      <c r="C43" s="77" t="s">
+      <c r="C43" s="76" t="s">
         <v>1763</v>
       </c>
-      <c r="D43" s="77"/>
-      <c r="E43" s="77"/>
-      <c r="F43" s="77"/>
-      <c r="G43" s="77"/>
-      <c r="H43" s="77"/>
+      <c r="D43" s="76"/>
+      <c r="E43" s="76"/>
+      <c r="F43" s="76"/>
+      <c r="G43" s="76"/>
+      <c r="H43" s="76"/>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" s="36" t="s">
@@ -17285,26 +17319,26 @@
       <c r="B44" s="28" t="s">
         <v>1740</v>
       </c>
-      <c r="C44" s="77" t="s">
+      <c r="C44" s="76" t="s">
         <v>1765</v>
       </c>
-      <c r="D44" s="77"/>
-      <c r="E44" s="77"/>
-      <c r="F44" s="77"/>
-      <c r="G44" s="77"/>
-      <c r="H44" s="77"/>
+      <c r="D44" s="76"/>
+      <c r="E44" s="76"/>
+      <c r="F44" s="76"/>
+      <c r="G44" s="76"/>
+      <c r="H44" s="76"/>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A48" s="78" t="s">
+      <c r="A48" s="75" t="s">
         <v>1754</v>
       </c>
-      <c r="B48" s="78"/>
-      <c r="C48" s="78"/>
-      <c r="D48" s="78"/>
-      <c r="E48" s="78"/>
-      <c r="F48" s="78"/>
-      <c r="G48" s="78"/>
-      <c r="H48" s="78"/>
+      <c r="B48" s="75"/>
+      <c r="C48" s="75"/>
+      <c r="D48" s="75"/>
+      <c r="E48" s="75"/>
+      <c r="F48" s="75"/>
+      <c r="G48" s="75"/>
+      <c r="H48" s="75"/>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
@@ -17317,16 +17351,16 @@
       </c>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A52" s="78" t="s">
+      <c r="A52" s="75" t="s">
         <v>1756</v>
       </c>
-      <c r="B52" s="78"/>
-      <c r="C52" s="78"/>
-      <c r="D52" s="78"/>
-      <c r="E52" s="78"/>
-      <c r="F52" s="78"/>
-      <c r="G52" s="78"/>
-      <c r="H52" s="78"/>
+      <c r="B52" s="75"/>
+      <c r="C52" s="75"/>
+      <c r="D52" s="75"/>
+      <c r="E52" s="75"/>
+      <c r="F52" s="75"/>
+      <c r="G52" s="75"/>
+      <c r="H52" s="75"/>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
@@ -17334,16 +17368,16 @@
       </c>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A57" s="78" t="s">
+      <c r="A57" s="75" t="s">
         <v>1769</v>
       </c>
-      <c r="B57" s="78"/>
-      <c r="C57" s="78"/>
-      <c r="D57" s="78"/>
-      <c r="E57" s="78"/>
-      <c r="F57" s="78"/>
-      <c r="G57" s="78"/>
-      <c r="H57" s="78"/>
+      <c r="B57" s="75"/>
+      <c r="C57" s="75"/>
+      <c r="D57" s="75"/>
+      <c r="E57" s="75"/>
+      <c r="F57" s="75"/>
+      <c r="G57" s="75"/>
+      <c r="H57" s="75"/>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
@@ -17411,12 +17445,12 @@
       </c>
     </row>
     <row r="73" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="H73" s="78" t="s">
+      <c r="H73" s="75" t="s">
         <v>1783</v>
       </c>
-      <c r="I73" s="78"/>
-      <c r="J73" s="78"/>
-      <c r="K73" s="78"/>
+      <c r="I73" s="75"/>
+      <c r="J73" s="75"/>
+      <c r="K73" s="75"/>
     </row>
     <row r="74" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A74" s="55" t="s">
@@ -17983,6 +18017,16 @@
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="C32:H32"/>
+    <mergeCell ref="C33:H33"/>
+    <mergeCell ref="C34:H34"/>
+    <mergeCell ref="C35:H35"/>
+    <mergeCell ref="C36:H36"/>
+    <mergeCell ref="C37:H37"/>
+    <mergeCell ref="C38:H38"/>
+    <mergeCell ref="C39:H39"/>
+    <mergeCell ref="C40:H40"/>
+    <mergeCell ref="C41:H41"/>
     <mergeCell ref="A57:H57"/>
     <mergeCell ref="H73:K73"/>
     <mergeCell ref="C42:H42"/>
@@ -17990,16 +18034,6 @@
     <mergeCell ref="C44:H44"/>
     <mergeCell ref="A48:H48"/>
     <mergeCell ref="A52:H52"/>
-    <mergeCell ref="C37:H37"/>
-    <mergeCell ref="C38:H38"/>
-    <mergeCell ref="C39:H39"/>
-    <mergeCell ref="C40:H40"/>
-    <mergeCell ref="C41:H41"/>
-    <mergeCell ref="C32:H32"/>
-    <mergeCell ref="C33:H33"/>
-    <mergeCell ref="C34:H34"/>
-    <mergeCell ref="C35:H35"/>
-    <mergeCell ref="C36:H36"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78749999999999998" bottom="0.78749999999999998" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -18062,13 +18096,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="78" t="s">
+      <c r="A1" s="75" t="s">
         <v>1905</v>
       </c>
-      <c r="B1" s="78"/>
-      <c r="C1" s="78"/>
-      <c r="D1" s="78"/>
-      <c r="E1" s="78"/>
+      <c r="B1" s="75"/>
+      <c r="C1" s="75"/>
+      <c r="D1" s="75"/>
+      <c r="E1" s="75"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="56" t="s">
@@ -18166,7 +18200,7 @@
 
 <file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1E00-000000000000}">
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:A11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
@@ -18217,6 +18251,11 @@
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>1922</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>2287</v>
       </c>
     </row>
   </sheetData>
@@ -22402,10 +22441,10 @@
         <v>2282</v>
       </c>
       <c r="D34" t="s">
+        <v>2288</v>
+      </c>
+      <c r="E34" t="s">
         <v>2283</v>
-      </c>
-      <c r="E34" t="s">
-        <v>2284</v>
       </c>
     </row>
   </sheetData>
@@ -22437,10 +22476,10 @@
       <c r="A4" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="C4" s="70" t="s">
+      <c r="C4" s="69" t="s">
         <v>50</v>
       </c>
-      <c r="D4" s="70"/>
+      <c r="D4" s="69"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
@@ -22482,10 +22521,10 @@
       <c r="A11" t="s">
         <v>59</v>
       </c>
-      <c r="C11" s="70" t="s">
+      <c r="C11" s="69" t="s">
         <v>60</v>
       </c>
-      <c r="D11" s="70"/>
+      <c r="D11" s="69"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
@@ -24320,11 +24359,11 @@
       <c r="D1" t="s">
         <v>393</v>
       </c>
-      <c r="F1" s="68" t="s">
+      <c r="F1" s="70" t="s">
         <v>400</v>
       </c>
-      <c r="G1" s="68"/>
-      <c r="H1" s="68"/>
+      <c r="G1" s="70"/>
+      <c r="H1" s="70"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2">

</xml_diff>

<commit_message>
Song 33 out of Music.amb until the remake supports it (Song 33 = Intro there), prototype uses song 22, remake screenshots
</commit_message>
<xml_diff>
--- a/AmbermoonAdvanced.xlsx
+++ b/AmbermoonAdvanced.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Robert\source\repos\Ambermoon-Advanced\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{715E6CB1-654C-47A9-B89E-A0331E10411F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CB8A306-860D-4B1E-9782-98590EF10961}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" firstSheet="36" activeTab="42" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7046,22 +7046,22 @@
     <t>-</t>
   </si>
   <si>
-    <t>New in Advanced. Song 22 starting and looping at position 34, positions 52-53 and the last 3 removed (about 60 s per loop). Source: assets/Temples/music/SONIC.PsychedelicDuneGroove_ab34_cut2. Code: Max_music = 33 in Set_music (the harp still shows 32 songs). Remake support missing.</t>
-  </si>
-  <si>
     <t>Palast des S'Riel (Prototyp) / Palace of S'Riel (prototype)</t>
   </si>
   <si>
-    <t>Temple rework pilot, only reachable with the cheat map jump (t, 487). Built by assets/Temples/tools/build_prototype.py. Labdata 46, palette 59, music 33. Exit to 520 (37,41) like 444. Reuses chests 116/117 of map 444.</t>
-  </si>
-  <si>
     <t>S'Riel prototype (487): copy of labdata 5 (Gala temple) with floor 20 and ceiling 8. Palette 59 (Sandstein) is new too.</t>
   </si>
   <si>
     <t>Add automaps 485 (27x27, 92 bytes), 486 (11x19, 27 bytes) and 487 (17x17, 37 bytes). They were missing in Save.00, entering 485/486 on the Amiga ends in a fatal error (Init_automap loads the entry for every 3D map).</t>
   </si>
   <si>
-    <t>Prototype map 487 (S'Riel); final temple open</t>
+    <t>Chosen as temple music, not in Music.amb yet</t>
+  </si>
+  <si>
+    <t>New in Advanced. Song 22 starting and looping at position 34, positions 52-53 and the last 3 removed (about 60 s per loop). Source: assets/Temples/music/SONIC.PsychedelicDuneGroove_ab34_cut2. Amiga code ready (Max_music = 33 in Set_music, the harp still shows 32 songs). NOT in Music.amb yet: in the remake Song 33 = Intro, a 33rd Music.amb entry makes the data loading fail. Append it after the remake is changed.</t>
+  </si>
+  <si>
+    <t>Temple rework pilot, only reachable with the cheat map jump (t, 487) or the remake teleport cheat. Built by assets/Temples/tools/build_prototype.py. Labdata 46, palette 59, music 22 (later 33). Exit to 520 (37,41) like 444. Reuses chests 116/117 of map 444.</t>
   </si>
 </sst>
 </file>
@@ -7707,17 +7707,17 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="21" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="27" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="27" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="21" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -9953,13 +9953,13 @@
         <v>487</v>
       </c>
       <c r="B48" t="s">
-        <v>2284</v>
+        <v>2283</v>
       </c>
       <c r="C48" t="s">
         <v>911</v>
       </c>
       <c r="D48" t="s">
-        <v>2285</v>
+        <v>2288</v>
       </c>
     </row>
   </sheetData>
@@ -10176,7 +10176,7 @@
         <v>46</v>
       </c>
       <c r="B14" t="s">
-        <v>2286</v>
+        <v>2284</v>
       </c>
     </row>
   </sheetData>
@@ -17127,14 +17127,14 @@
       <c r="B32" s="54" t="s">
         <v>1745</v>
       </c>
-      <c r="C32" s="78" t="s">
+      <c r="C32" s="75" t="s">
         <v>1746</v>
       </c>
-      <c r="D32" s="78"/>
-      <c r="E32" s="78"/>
-      <c r="F32" s="78"/>
-      <c r="G32" s="78"/>
-      <c r="H32" s="78"/>
+      <c r="D32" s="75"/>
+      <c r="E32" s="75"/>
+      <c r="F32" s="75"/>
+      <c r="G32" s="75"/>
+      <c r="H32" s="75"/>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" s="36" t="s">
@@ -17143,14 +17143,14 @@
       <c r="B33" s="28" t="s">
         <v>1748</v>
       </c>
-      <c r="C33" s="77" t="s">
+      <c r="C33" s="76" t="s">
         <v>1749</v>
       </c>
-      <c r="D33" s="77"/>
-      <c r="E33" s="77"/>
-      <c r="F33" s="77"/>
-      <c r="G33" s="77"/>
-      <c r="H33" s="77"/>
+      <c r="D33" s="76"/>
+      <c r="E33" s="76"/>
+      <c r="F33" s="76"/>
+      <c r="G33" s="76"/>
+      <c r="H33" s="76"/>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" s="36" t="s">
@@ -17159,14 +17159,14 @@
       <c r="B34" s="28" t="s">
         <v>1748</v>
       </c>
-      <c r="C34" s="77" t="s">
+      <c r="C34" s="76" t="s">
         <v>1749</v>
       </c>
-      <c r="D34" s="77"/>
-      <c r="E34" s="77"/>
-      <c r="F34" s="77"/>
-      <c r="G34" s="77"/>
-      <c r="H34" s="77"/>
+      <c r="D34" s="76"/>
+      <c r="E34" s="76"/>
+      <c r="F34" s="76"/>
+      <c r="G34" s="76"/>
+      <c r="H34" s="76"/>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" s="36" t="s">
@@ -17175,14 +17175,14 @@
       <c r="B35" s="28" t="s">
         <v>1748</v>
       </c>
-      <c r="C35" s="77" t="s">
+      <c r="C35" s="76" t="s">
         <v>1749</v>
       </c>
-      <c r="D35" s="77"/>
-      <c r="E35" s="77"/>
-      <c r="F35" s="77"/>
-      <c r="G35" s="77"/>
-      <c r="H35" s="77"/>
+      <c r="D35" s="76"/>
+      <c r="E35" s="76"/>
+      <c r="F35" s="76"/>
+      <c r="G35" s="76"/>
+      <c r="H35" s="76"/>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" s="36" t="s">
@@ -17191,14 +17191,14 @@
       <c r="B36" s="28" t="s">
         <v>1734</v>
       </c>
-      <c r="C36" s="76" t="s">
+      <c r="C36" s="77" t="s">
         <v>1753</v>
       </c>
-      <c r="D36" s="76"/>
-      <c r="E36" s="76"/>
-      <c r="F36" s="76"/>
-      <c r="G36" s="76"/>
-      <c r="H36" s="76"/>
+      <c r="D36" s="77"/>
+      <c r="E36" s="77"/>
+      <c r="F36" s="77"/>
+      <c r="G36" s="77"/>
+      <c r="H36" s="77"/>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" s="36" t="s">
@@ -17207,14 +17207,14 @@
       <c r="B37" s="28" t="s">
         <v>1736</v>
       </c>
-      <c r="C37" s="77" t="s">
+      <c r="C37" s="76" t="s">
         <v>1755</v>
       </c>
-      <c r="D37" s="77"/>
-      <c r="E37" s="77"/>
-      <c r="F37" s="77"/>
-      <c r="G37" s="77"/>
-      <c r="H37" s="77"/>
+      <c r="D37" s="76"/>
+      <c r="E37" s="76"/>
+      <c r="F37" s="76"/>
+      <c r="G37" s="76"/>
+      <c r="H37" s="76"/>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" s="36" t="s">
@@ -17223,14 +17223,14 @@
       <c r="B38" s="28" t="s">
         <v>1734</v>
       </c>
-      <c r="C38" s="77" t="s">
+      <c r="C38" s="76" t="s">
         <v>1755</v>
       </c>
-      <c r="D38" s="77"/>
-      <c r="E38" s="77"/>
-      <c r="F38" s="77"/>
-      <c r="G38" s="77"/>
-      <c r="H38" s="77"/>
+      <c r="D38" s="76"/>
+      <c r="E38" s="76"/>
+      <c r="F38" s="76"/>
+      <c r="G38" s="76"/>
+      <c r="H38" s="76"/>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" s="36" t="s">
@@ -17239,14 +17239,14 @@
       <c r="B39" s="28" t="s">
         <v>1734</v>
       </c>
-      <c r="C39" s="76" t="s">
+      <c r="C39" s="77" t="s">
         <v>1753</v>
       </c>
-      <c r="D39" s="76"/>
-      <c r="E39" s="76"/>
-      <c r="F39" s="76"/>
-      <c r="G39" s="76"/>
-      <c r="H39" s="76"/>
+      <c r="D39" s="77"/>
+      <c r="E39" s="77"/>
+      <c r="F39" s="77"/>
+      <c r="G39" s="77"/>
+      <c r="H39" s="77"/>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" s="36" t="s">
@@ -17255,14 +17255,14 @@
       <c r="B40" s="28" t="s">
         <v>1734</v>
       </c>
-      <c r="C40" s="76" t="s">
+      <c r="C40" s="77" t="s">
         <v>1753</v>
       </c>
-      <c r="D40" s="76"/>
-      <c r="E40" s="76"/>
-      <c r="F40" s="76"/>
-      <c r="G40" s="76"/>
-      <c r="H40" s="76"/>
+      <c r="D40" s="77"/>
+      <c r="E40" s="77"/>
+      <c r="F40" s="77"/>
+      <c r="G40" s="77"/>
+      <c r="H40" s="77"/>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" s="36" t="s">
@@ -17271,14 +17271,14 @@
       <c r="B41" s="28" t="s">
         <v>1737</v>
       </c>
-      <c r="C41" s="76" t="s">
+      <c r="C41" s="77" t="s">
         <v>1759</v>
       </c>
-      <c r="D41" s="76"/>
-      <c r="E41" s="76"/>
-      <c r="F41" s="76"/>
-      <c r="G41" s="76"/>
-      <c r="H41" s="76"/>
+      <c r="D41" s="77"/>
+      <c r="E41" s="77"/>
+      <c r="F41" s="77"/>
+      <c r="G41" s="77"/>
+      <c r="H41" s="77"/>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" s="36" t="s">
@@ -17287,14 +17287,14 @@
       <c r="B42" s="28" t="s">
         <v>1738</v>
       </c>
-      <c r="C42" s="76" t="s">
+      <c r="C42" s="77" t="s">
         <v>1761</v>
       </c>
-      <c r="D42" s="76"/>
-      <c r="E42" s="76"/>
-      <c r="F42" s="76"/>
-      <c r="G42" s="76"/>
-      <c r="H42" s="76"/>
+      <c r="D42" s="77"/>
+      <c r="E42" s="77"/>
+      <c r="F42" s="77"/>
+      <c r="G42" s="77"/>
+      <c r="H42" s="77"/>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" s="36" t="s">
@@ -17303,14 +17303,14 @@
       <c r="B43" s="28" t="s">
         <v>1739</v>
       </c>
-      <c r="C43" s="76" t="s">
+      <c r="C43" s="77" t="s">
         <v>1763</v>
       </c>
-      <c r="D43" s="76"/>
-      <c r="E43" s="76"/>
-      <c r="F43" s="76"/>
-      <c r="G43" s="76"/>
-      <c r="H43" s="76"/>
+      <c r="D43" s="77"/>
+      <c r="E43" s="77"/>
+      <c r="F43" s="77"/>
+      <c r="G43" s="77"/>
+      <c r="H43" s="77"/>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" s="36" t="s">
@@ -17319,26 +17319,26 @@
       <c r="B44" s="28" t="s">
         <v>1740</v>
       </c>
-      <c r="C44" s="76" t="s">
+      <c r="C44" s="77" t="s">
         <v>1765</v>
       </c>
-      <c r="D44" s="76"/>
-      <c r="E44" s="76"/>
-      <c r="F44" s="76"/>
-      <c r="G44" s="76"/>
-      <c r="H44" s="76"/>
+      <c r="D44" s="77"/>
+      <c r="E44" s="77"/>
+      <c r="F44" s="77"/>
+      <c r="G44" s="77"/>
+      <c r="H44" s="77"/>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A48" s="75" t="s">
+      <c r="A48" s="78" t="s">
         <v>1754</v>
       </c>
-      <c r="B48" s="75"/>
-      <c r="C48" s="75"/>
-      <c r="D48" s="75"/>
-      <c r="E48" s="75"/>
-      <c r="F48" s="75"/>
-      <c r="G48" s="75"/>
-      <c r="H48" s="75"/>
+      <c r="B48" s="78"/>
+      <c r="C48" s="78"/>
+      <c r="D48" s="78"/>
+      <c r="E48" s="78"/>
+      <c r="F48" s="78"/>
+      <c r="G48" s="78"/>
+      <c r="H48" s="78"/>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
@@ -17351,16 +17351,16 @@
       </c>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A52" s="75" t="s">
+      <c r="A52" s="78" t="s">
         <v>1756</v>
       </c>
-      <c r="B52" s="75"/>
-      <c r="C52" s="75"/>
-      <c r="D52" s="75"/>
-      <c r="E52" s="75"/>
-      <c r="F52" s="75"/>
-      <c r="G52" s="75"/>
-      <c r="H52" s="75"/>
+      <c r="B52" s="78"/>
+      <c r="C52" s="78"/>
+      <c r="D52" s="78"/>
+      <c r="E52" s="78"/>
+      <c r="F52" s="78"/>
+      <c r="G52" s="78"/>
+      <c r="H52" s="78"/>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
@@ -17368,16 +17368,16 @@
       </c>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A57" s="75" t="s">
+      <c r="A57" s="78" t="s">
         <v>1769</v>
       </c>
-      <c r="B57" s="75"/>
-      <c r="C57" s="75"/>
-      <c r="D57" s="75"/>
-      <c r="E57" s="75"/>
-      <c r="F57" s="75"/>
-      <c r="G57" s="75"/>
-      <c r="H57" s="75"/>
+      <c r="B57" s="78"/>
+      <c r="C57" s="78"/>
+      <c r="D57" s="78"/>
+      <c r="E57" s="78"/>
+      <c r="F57" s="78"/>
+      <c r="G57" s="78"/>
+      <c r="H57" s="78"/>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
@@ -17445,12 +17445,12 @@
       </c>
     </row>
     <row r="73" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="H73" s="75" t="s">
+      <c r="H73" s="78" t="s">
         <v>1783</v>
       </c>
-      <c r="I73" s="75"/>
-      <c r="J73" s="75"/>
-      <c r="K73" s="75"/>
+      <c r="I73" s="78"/>
+      <c r="J73" s="78"/>
+      <c r="K73" s="78"/>
     </row>
     <row r="74" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A74" s="55" t="s">
@@ -18017,16 +18017,6 @@
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="C32:H32"/>
-    <mergeCell ref="C33:H33"/>
-    <mergeCell ref="C34:H34"/>
-    <mergeCell ref="C35:H35"/>
-    <mergeCell ref="C36:H36"/>
-    <mergeCell ref="C37:H37"/>
-    <mergeCell ref="C38:H38"/>
-    <mergeCell ref="C39:H39"/>
-    <mergeCell ref="C40:H40"/>
-    <mergeCell ref="C41:H41"/>
     <mergeCell ref="A57:H57"/>
     <mergeCell ref="H73:K73"/>
     <mergeCell ref="C42:H42"/>
@@ -18034,6 +18024,16 @@
     <mergeCell ref="C44:H44"/>
     <mergeCell ref="A48:H48"/>
     <mergeCell ref="A52:H52"/>
+    <mergeCell ref="C37:H37"/>
+    <mergeCell ref="C38:H38"/>
+    <mergeCell ref="C39:H39"/>
+    <mergeCell ref="C40:H40"/>
+    <mergeCell ref="C41:H41"/>
+    <mergeCell ref="C32:H32"/>
+    <mergeCell ref="C33:H33"/>
+    <mergeCell ref="C34:H34"/>
+    <mergeCell ref="C35:H35"/>
+    <mergeCell ref="C36:H36"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78749999999999998" bottom="0.78749999999999998" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -18096,13 +18096,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="75" t="s">
+      <c r="A1" s="78" t="s">
         <v>1905</v>
       </c>
-      <c r="B1" s="75"/>
-      <c r="C1" s="75"/>
-      <c r="D1" s="75"/>
-      <c r="E1" s="75"/>
+      <c r="B1" s="78"/>
+      <c r="C1" s="78"/>
+      <c r="D1" s="78"/>
+      <c r="E1" s="78"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="56" t="s">
@@ -18255,7 +18255,7 @@
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>2287</v>
+        <v>2285</v>
       </c>
     </row>
   </sheetData>
@@ -22441,10 +22441,10 @@
         <v>2282</v>
       </c>
       <c r="D34" t="s">
-        <v>2288</v>
+        <v>2286</v>
       </c>
       <c r="E34" t="s">
-        <v>2283</v>
+        <v>2287</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Sandstone temple walls 193-195 from the new texture, palette 59 Wüstentempel, S'Riel prototype uses them, PNG reader/downscale/quantize in textures.py
</commit_message>
<xml_diff>
--- a/AmbermoonAdvanced.xlsx
+++ b/AmbermoonAdvanced.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Robert\source\repos\Ambermoon-Advanced\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CB8A306-860D-4B1E-9782-98590EF10961}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52AEAF11-B256-4B21-AE61-D4274FE27C3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" firstSheet="36" activeTab="42" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -78,7 +78,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3181" uniqueCount="2289">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3190" uniqueCount="2293">
   <si>
     <t>Map texts</t>
   </si>
@@ -7049,9 +7049,6 @@
     <t>Palast des S'Riel (Prototyp) / Palace of S'Riel (prototype)</t>
   </si>
   <si>
-    <t>S'Riel prototype (487): copy of labdata 5 (Gala temple) with floor 20 and ceiling 8. Palette 59 (Sandstein) is new too.</t>
-  </si>
-  <si>
     <t>Add automaps 485 (27x27, 92 bytes), 486 (11x19, 27 bytes) and 487 (17x17, 37 bytes). They were missing in Save.00, entering 485/486 on the Amiga ends in a fatal error (Init_automap loads the entry for every 3D map).</t>
   </si>
   <si>
@@ -7062,6 +7059,21 @@
   </si>
   <si>
     <t>Temple rework pilot, only reachable with the cheat map jump (t, 487) or the remake teleport cheat. Built by assets/Temples/tools/build_prototype.py. Labdata 46, palette 59, music 22 (later 33). Exit to 520 (37,41) like 444. Reuses chests 116/117 of map 444.</t>
+  </si>
+  <si>
+    <t>Sandstone wall with friezes and two lotus columns</t>
+  </si>
+  <si>
+    <t>Temple prototype S'Riel (487)</t>
+  </si>
+  <si>
+    <t>Sandstone wall with friezes, no columns (base for window, crest, rosette and painting overlays)</t>
+  </si>
+  <si>
+    <t>Sandstone gateway (dark passage between the columns, passable)</t>
+  </si>
+  <si>
+    <t>S'Riel prototype (487): copy of labdata 5 (Gala temple) with floor 20, ceiling 8 and the new walls 131-138 (sandstone textures 193-195; 134-138 are 194 with the overlays window 72, crest 74, painting 67, rosette 71, painting 68). Palette 59 (Wüstentempel) is new too.</t>
   </si>
 </sst>
 </file>
@@ -7707,17 +7719,17 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="27" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="21" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="27" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="21" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -9959,7 +9971,7 @@
         <v>911</v>
       </c>
       <c r="D48" t="s">
-        <v>2288</v>
+        <v>2287</v>
       </c>
     </row>
   </sheetData>
@@ -10176,7 +10188,7 @@
         <v>46</v>
       </c>
       <c r="B14" t="s">
-        <v>2284</v>
+        <v>2292</v>
       </c>
     </row>
   </sheetData>
@@ -14662,7 +14674,7 @@
 
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1500-000000000000}">
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="67.85546875" customWidth="1"/>
@@ -14960,6 +14972,48 @@
         <v>1520</v>
       </c>
       <c r="D21" t="s">
+        <v>1530</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>193</v>
+      </c>
+      <c r="B22" t="s">
+        <v>2288</v>
+      </c>
+      <c r="C22" t="s">
+        <v>2289</v>
+      </c>
+      <c r="D22" t="s">
+        <v>1530</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>194</v>
+      </c>
+      <c r="B23" t="s">
+        <v>2290</v>
+      </c>
+      <c r="C23" t="s">
+        <v>2289</v>
+      </c>
+      <c r="D23" t="s">
+        <v>1530</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>195</v>
+      </c>
+      <c r="B24" t="s">
+        <v>2291</v>
+      </c>
+      <c r="C24" t="s">
+        <v>2289</v>
+      </c>
+      <c r="D24" t="s">
         <v>1530</v>
       </c>
     </row>
@@ -17127,14 +17181,14 @@
       <c r="B32" s="54" t="s">
         <v>1745</v>
       </c>
-      <c r="C32" s="75" t="s">
+      <c r="C32" s="78" t="s">
         <v>1746</v>
       </c>
-      <c r="D32" s="75"/>
-      <c r="E32" s="75"/>
-      <c r="F32" s="75"/>
-      <c r="G32" s="75"/>
-      <c r="H32" s="75"/>
+      <c r="D32" s="78"/>
+      <c r="E32" s="78"/>
+      <c r="F32" s="78"/>
+      <c r="G32" s="78"/>
+      <c r="H32" s="78"/>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" s="36" t="s">
@@ -17143,14 +17197,14 @@
       <c r="B33" s="28" t="s">
         <v>1748</v>
       </c>
-      <c r="C33" s="76" t="s">
+      <c r="C33" s="77" t="s">
         <v>1749</v>
       </c>
-      <c r="D33" s="76"/>
-      <c r="E33" s="76"/>
-      <c r="F33" s="76"/>
-      <c r="G33" s="76"/>
-      <c r="H33" s="76"/>
+      <c r="D33" s="77"/>
+      <c r="E33" s="77"/>
+      <c r="F33" s="77"/>
+      <c r="G33" s="77"/>
+      <c r="H33" s="77"/>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" s="36" t="s">
@@ -17159,14 +17213,14 @@
       <c r="B34" s="28" t="s">
         <v>1748</v>
       </c>
-      <c r="C34" s="76" t="s">
+      <c r="C34" s="77" t="s">
         <v>1749</v>
       </c>
-      <c r="D34" s="76"/>
-      <c r="E34" s="76"/>
-      <c r="F34" s="76"/>
-      <c r="G34" s="76"/>
-      <c r="H34" s="76"/>
+      <c r="D34" s="77"/>
+      <c r="E34" s="77"/>
+      <c r="F34" s="77"/>
+      <c r="G34" s="77"/>
+      <c r="H34" s="77"/>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" s="36" t="s">
@@ -17175,14 +17229,14 @@
       <c r="B35" s="28" t="s">
         <v>1748</v>
       </c>
-      <c r="C35" s="76" t="s">
+      <c r="C35" s="77" t="s">
         <v>1749</v>
       </c>
-      <c r="D35" s="76"/>
-      <c r="E35" s="76"/>
-      <c r="F35" s="76"/>
-      <c r="G35" s="76"/>
-      <c r="H35" s="76"/>
+      <c r="D35" s="77"/>
+      <c r="E35" s="77"/>
+      <c r="F35" s="77"/>
+      <c r="G35" s="77"/>
+      <c r="H35" s="77"/>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" s="36" t="s">
@@ -17191,14 +17245,14 @@
       <c r="B36" s="28" t="s">
         <v>1734</v>
       </c>
-      <c r="C36" s="77" t="s">
+      <c r="C36" s="76" t="s">
         <v>1753</v>
       </c>
-      <c r="D36" s="77"/>
-      <c r="E36" s="77"/>
-      <c r="F36" s="77"/>
-      <c r="G36" s="77"/>
-      <c r="H36" s="77"/>
+      <c r="D36" s="76"/>
+      <c r="E36" s="76"/>
+      <c r="F36" s="76"/>
+      <c r="G36" s="76"/>
+      <c r="H36" s="76"/>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" s="36" t="s">
@@ -17207,14 +17261,14 @@
       <c r="B37" s="28" t="s">
         <v>1736</v>
       </c>
-      <c r="C37" s="76" t="s">
+      <c r="C37" s="77" t="s">
         <v>1755</v>
       </c>
-      <c r="D37" s="76"/>
-      <c r="E37" s="76"/>
-      <c r="F37" s="76"/>
-      <c r="G37" s="76"/>
-      <c r="H37" s="76"/>
+      <c r="D37" s="77"/>
+      <c r="E37" s="77"/>
+      <c r="F37" s="77"/>
+      <c r="G37" s="77"/>
+      <c r="H37" s="77"/>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" s="36" t="s">
@@ -17223,14 +17277,14 @@
       <c r="B38" s="28" t="s">
         <v>1734</v>
       </c>
-      <c r="C38" s="76" t="s">
+      <c r="C38" s="77" t="s">
         <v>1755</v>
       </c>
-      <c r="D38" s="76"/>
-      <c r="E38" s="76"/>
-      <c r="F38" s="76"/>
-      <c r="G38" s="76"/>
-      <c r="H38" s="76"/>
+      <c r="D38" s="77"/>
+      <c r="E38" s="77"/>
+      <c r="F38" s="77"/>
+      <c r="G38" s="77"/>
+      <c r="H38" s="77"/>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" s="36" t="s">
@@ -17239,14 +17293,14 @@
       <c r="B39" s="28" t="s">
         <v>1734</v>
       </c>
-      <c r="C39" s="77" t="s">
+      <c r="C39" s="76" t="s">
         <v>1753</v>
       </c>
-      <c r="D39" s="77"/>
-      <c r="E39" s="77"/>
-      <c r="F39" s="77"/>
-      <c r="G39" s="77"/>
-      <c r="H39" s="77"/>
+      <c r="D39" s="76"/>
+      <c r="E39" s="76"/>
+      <c r="F39" s="76"/>
+      <c r="G39" s="76"/>
+      <c r="H39" s="76"/>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" s="36" t="s">
@@ -17255,14 +17309,14 @@
       <c r="B40" s="28" t="s">
         <v>1734</v>
       </c>
-      <c r="C40" s="77" t="s">
+      <c r="C40" s="76" t="s">
         <v>1753</v>
       </c>
-      <c r="D40" s="77"/>
-      <c r="E40" s="77"/>
-      <c r="F40" s="77"/>
-      <c r="G40" s="77"/>
-      <c r="H40" s="77"/>
+      <c r="D40" s="76"/>
+      <c r="E40" s="76"/>
+      <c r="F40" s="76"/>
+      <c r="G40" s="76"/>
+      <c r="H40" s="76"/>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" s="36" t="s">
@@ -17271,14 +17325,14 @@
       <c r="B41" s="28" t="s">
         <v>1737</v>
       </c>
-      <c r="C41" s="77" t="s">
+      <c r="C41" s="76" t="s">
         <v>1759</v>
       </c>
-      <c r="D41" s="77"/>
-      <c r="E41" s="77"/>
-      <c r="F41" s="77"/>
-      <c r="G41" s="77"/>
-      <c r="H41" s="77"/>
+      <c r="D41" s="76"/>
+      <c r="E41" s="76"/>
+      <c r="F41" s="76"/>
+      <c r="G41" s="76"/>
+      <c r="H41" s="76"/>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" s="36" t="s">
@@ -17287,14 +17341,14 @@
       <c r="B42" s="28" t="s">
         <v>1738</v>
       </c>
-      <c r="C42" s="77" t="s">
+      <c r="C42" s="76" t="s">
         <v>1761</v>
       </c>
-      <c r="D42" s="77"/>
-      <c r="E42" s="77"/>
-      <c r="F42" s="77"/>
-      <c r="G42" s="77"/>
-      <c r="H42" s="77"/>
+      <c r="D42" s="76"/>
+      <c r="E42" s="76"/>
+      <c r="F42" s="76"/>
+      <c r="G42" s="76"/>
+      <c r="H42" s="76"/>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" s="36" t="s">
@@ -17303,14 +17357,14 @@
       <c r="B43" s="28" t="s">
         <v>1739</v>
       </c>
-      <c r="C43" s="77" t="s">
+      <c r="C43" s="76" t="s">
         <v>1763</v>
       </c>
-      <c r="D43" s="77"/>
-      <c r="E43" s="77"/>
-      <c r="F43" s="77"/>
-      <c r="G43" s="77"/>
-      <c r="H43" s="77"/>
+      <c r="D43" s="76"/>
+      <c r="E43" s="76"/>
+      <c r="F43" s="76"/>
+      <c r="G43" s="76"/>
+      <c r="H43" s="76"/>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" s="36" t="s">
@@ -17319,26 +17373,26 @@
       <c r="B44" s="28" t="s">
         <v>1740</v>
       </c>
-      <c r="C44" s="77" t="s">
+      <c r="C44" s="76" t="s">
         <v>1765</v>
       </c>
-      <c r="D44" s="77"/>
-      <c r="E44" s="77"/>
-      <c r="F44" s="77"/>
-      <c r="G44" s="77"/>
-      <c r="H44" s="77"/>
+      <c r="D44" s="76"/>
+      <c r="E44" s="76"/>
+      <c r="F44" s="76"/>
+      <c r="G44" s="76"/>
+      <c r="H44" s="76"/>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A48" s="78" t="s">
+      <c r="A48" s="75" t="s">
         <v>1754</v>
       </c>
-      <c r="B48" s="78"/>
-      <c r="C48" s="78"/>
-      <c r="D48" s="78"/>
-      <c r="E48" s="78"/>
-      <c r="F48" s="78"/>
-      <c r="G48" s="78"/>
-      <c r="H48" s="78"/>
+      <c r="B48" s="75"/>
+      <c r="C48" s="75"/>
+      <c r="D48" s="75"/>
+      <c r="E48" s="75"/>
+      <c r="F48" s="75"/>
+      <c r="G48" s="75"/>
+      <c r="H48" s="75"/>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
@@ -17351,16 +17405,16 @@
       </c>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A52" s="78" t="s">
+      <c r="A52" s="75" t="s">
         <v>1756</v>
       </c>
-      <c r="B52" s="78"/>
-      <c r="C52" s="78"/>
-      <c r="D52" s="78"/>
-      <c r="E52" s="78"/>
-      <c r="F52" s="78"/>
-      <c r="G52" s="78"/>
-      <c r="H52" s="78"/>
+      <c r="B52" s="75"/>
+      <c r="C52" s="75"/>
+      <c r="D52" s="75"/>
+      <c r="E52" s="75"/>
+      <c r="F52" s="75"/>
+      <c r="G52" s="75"/>
+      <c r="H52" s="75"/>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
@@ -17368,16 +17422,16 @@
       </c>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A57" s="78" t="s">
+      <c r="A57" s="75" t="s">
         <v>1769</v>
       </c>
-      <c r="B57" s="78"/>
-      <c r="C57" s="78"/>
-      <c r="D57" s="78"/>
-      <c r="E57" s="78"/>
-      <c r="F57" s="78"/>
-      <c r="G57" s="78"/>
-      <c r="H57" s="78"/>
+      <c r="B57" s="75"/>
+      <c r="C57" s="75"/>
+      <c r="D57" s="75"/>
+      <c r="E57" s="75"/>
+      <c r="F57" s="75"/>
+      <c r="G57" s="75"/>
+      <c r="H57" s="75"/>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
@@ -17445,12 +17499,12 @@
       </c>
     </row>
     <row r="73" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="H73" s="78" t="s">
+      <c r="H73" s="75" t="s">
         <v>1783</v>
       </c>
-      <c r="I73" s="78"/>
-      <c r="J73" s="78"/>
-      <c r="K73" s="78"/>
+      <c r="I73" s="75"/>
+      <c r="J73" s="75"/>
+      <c r="K73" s="75"/>
     </row>
     <row r="74" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A74" s="55" t="s">
@@ -18017,6 +18071,16 @@
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="C32:H32"/>
+    <mergeCell ref="C33:H33"/>
+    <mergeCell ref="C34:H34"/>
+    <mergeCell ref="C35:H35"/>
+    <mergeCell ref="C36:H36"/>
+    <mergeCell ref="C37:H37"/>
+    <mergeCell ref="C38:H38"/>
+    <mergeCell ref="C39:H39"/>
+    <mergeCell ref="C40:H40"/>
+    <mergeCell ref="C41:H41"/>
     <mergeCell ref="A57:H57"/>
     <mergeCell ref="H73:K73"/>
     <mergeCell ref="C42:H42"/>
@@ -18024,16 +18088,6 @@
     <mergeCell ref="C44:H44"/>
     <mergeCell ref="A48:H48"/>
     <mergeCell ref="A52:H52"/>
-    <mergeCell ref="C37:H37"/>
-    <mergeCell ref="C38:H38"/>
-    <mergeCell ref="C39:H39"/>
-    <mergeCell ref="C40:H40"/>
-    <mergeCell ref="C41:H41"/>
-    <mergeCell ref="C32:H32"/>
-    <mergeCell ref="C33:H33"/>
-    <mergeCell ref="C34:H34"/>
-    <mergeCell ref="C35:H35"/>
-    <mergeCell ref="C36:H36"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78749999999999998" bottom="0.78749999999999998" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -18096,13 +18150,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="78" t="s">
+      <c r="A1" s="75" t="s">
         <v>1905</v>
       </c>
-      <c r="B1" s="78"/>
-      <c r="C1" s="78"/>
-      <c r="D1" s="78"/>
-      <c r="E1" s="78"/>
+      <c r="B1" s="75"/>
+      <c r="C1" s="75"/>
+      <c r="D1" s="75"/>
+      <c r="E1" s="75"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="56" t="s">
@@ -18255,7 +18309,7 @@
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>2285</v>
+        <v>2284</v>
       </c>
     </row>
   </sheetData>
@@ -22441,10 +22495,10 @@
         <v>2282</v>
       </c>
       <c r="D34" t="s">
+        <v>2285</v>
+      </c>
+      <c r="E34" t="s">
         <v>2286</v>
-      </c>
-      <c r="E34" t="s">
-        <v>2287</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Temple base: labdata 46 = Gala walls + overlays (new walls 131-134 with column frames) in palette 59 'Wüstentempel' with more colour variance, sandstone textures 193-195 removed from the game data, Labdata 46.md
</commit_message>
<xml_diff>
--- a/AmbermoonAdvanced.xlsx
+++ b/AmbermoonAdvanced.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Robert\source\repos\Ambermoon-Advanced\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52AEAF11-B256-4B21-AE61-D4274FE27C3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E14F54B-0700-4FE1-A2FA-2CA5868C6A49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" firstSheet="36" activeTab="42" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -78,7 +78,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3190" uniqueCount="2293">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3181" uniqueCount="2289">
   <si>
     <t>Map texts</t>
   </si>
@@ -7061,19 +7061,7 @@
     <t>Temple rework pilot, only reachable with the cheat map jump (t, 487) or the remake teleport cheat. Built by assets/Temples/tools/build_prototype.py. Labdata 46, palette 59, music 22 (later 33). Exit to 520 (37,41) like 444. Reuses chests 116/117 of map 444.</t>
   </si>
   <si>
-    <t>Sandstone wall with friezes and two lotus columns</t>
-  </si>
-  <si>
-    <t>Temple prototype S'Riel (487)</t>
-  </si>
-  <si>
-    <t>Sandstone wall with friezes, no columns (base for window, crest, rosette and painting overlays)</t>
-  </si>
-  <si>
-    <t>Sandstone gateway (dark passage between the columns, passable)</t>
-  </si>
-  <si>
-    <t>S'Riel prototype (487): copy of labdata 5 (Gala temple) with floor 20, ceiling 8 and the new walls 131-138 (sandstone textures 193-195; 134-138 are 194 with the overlays window 72, crest 74, painting 67, rosette 71, painting 68). Palette 59 (Wüstentempel) is new too.</t>
+    <t>Temple base (first used by the S'Riel prototype, map 487): copy of labdata 5 (Gala temple) with floor 20, ceiling 8, new walls 131-134 (wall 99 with column frames 24/25 and rosette 71 / window 72 / crest 74) and object group 40 (serpent totem, texture 28). With palette 59 'Wüstentempel' (stone colours as sandstone, same index meaning as palette 6) everything turns into sandstone. Details: assets/Temples/Labdata 46.md</t>
   </si>
 </sst>
 </file>
@@ -7719,17 +7707,17 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="21" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="27" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="27" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="21" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -10188,7 +10176,7 @@
         <v>46</v>
       </c>
       <c r="B14" t="s">
-        <v>2292</v>
+        <v>2288</v>
       </c>
     </row>
   </sheetData>
@@ -14674,7 +14662,7 @@
 
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1500-000000000000}">
-  <dimension ref="A1:D24"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="67.85546875" customWidth="1"/>
@@ -14972,48 +14960,6 @@
         <v>1520</v>
       </c>
       <c r="D21" t="s">
-        <v>1530</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22">
-        <v>193</v>
-      </c>
-      <c r="B22" t="s">
-        <v>2288</v>
-      </c>
-      <c r="C22" t="s">
-        <v>2289</v>
-      </c>
-      <c r="D22" t="s">
-        <v>1530</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23">
-        <v>194</v>
-      </c>
-      <c r="B23" t="s">
-        <v>2290</v>
-      </c>
-      <c r="C23" t="s">
-        <v>2289</v>
-      </c>
-      <c r="D23" t="s">
-        <v>1530</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24">
-        <v>195</v>
-      </c>
-      <c r="B24" t="s">
-        <v>2291</v>
-      </c>
-      <c r="C24" t="s">
-        <v>2289</v>
-      </c>
-      <c r="D24" t="s">
         <v>1530</v>
       </c>
     </row>
@@ -17181,14 +17127,14 @@
       <c r="B32" s="54" t="s">
         <v>1745</v>
       </c>
-      <c r="C32" s="78" t="s">
+      <c r="C32" s="75" t="s">
         <v>1746</v>
       </c>
-      <c r="D32" s="78"/>
-      <c r="E32" s="78"/>
-      <c r="F32" s="78"/>
-      <c r="G32" s="78"/>
-      <c r="H32" s="78"/>
+      <c r="D32" s="75"/>
+      <c r="E32" s="75"/>
+      <c r="F32" s="75"/>
+      <c r="G32" s="75"/>
+      <c r="H32" s="75"/>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" s="36" t="s">
@@ -17197,14 +17143,14 @@
       <c r="B33" s="28" t="s">
         <v>1748</v>
       </c>
-      <c r="C33" s="77" t="s">
+      <c r="C33" s="76" t="s">
         <v>1749</v>
       </c>
-      <c r="D33" s="77"/>
-      <c r="E33" s="77"/>
-      <c r="F33" s="77"/>
-      <c r="G33" s="77"/>
-      <c r="H33" s="77"/>
+      <c r="D33" s="76"/>
+      <c r="E33" s="76"/>
+      <c r="F33" s="76"/>
+      <c r="G33" s="76"/>
+      <c r="H33" s="76"/>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" s="36" t="s">
@@ -17213,14 +17159,14 @@
       <c r="B34" s="28" t="s">
         <v>1748</v>
       </c>
-      <c r="C34" s="77" t="s">
+      <c r="C34" s="76" t="s">
         <v>1749</v>
       </c>
-      <c r="D34" s="77"/>
-      <c r="E34" s="77"/>
-      <c r="F34" s="77"/>
-      <c r="G34" s="77"/>
-      <c r="H34" s="77"/>
+      <c r="D34" s="76"/>
+      <c r="E34" s="76"/>
+      <c r="F34" s="76"/>
+      <c r="G34" s="76"/>
+      <c r="H34" s="76"/>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" s="36" t="s">
@@ -17229,14 +17175,14 @@
       <c r="B35" s="28" t="s">
         <v>1748</v>
       </c>
-      <c r="C35" s="77" t="s">
+      <c r="C35" s="76" t="s">
         <v>1749</v>
       </c>
-      <c r="D35" s="77"/>
-      <c r="E35" s="77"/>
-      <c r="F35" s="77"/>
-      <c r="G35" s="77"/>
-      <c r="H35" s="77"/>
+      <c r="D35" s="76"/>
+      <c r="E35" s="76"/>
+      <c r="F35" s="76"/>
+      <c r="G35" s="76"/>
+      <c r="H35" s="76"/>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" s="36" t="s">
@@ -17245,14 +17191,14 @@
       <c r="B36" s="28" t="s">
         <v>1734</v>
       </c>
-      <c r="C36" s="76" t="s">
+      <c r="C36" s="77" t="s">
         <v>1753</v>
       </c>
-      <c r="D36" s="76"/>
-      <c r="E36" s="76"/>
-      <c r="F36" s="76"/>
-      <c r="G36" s="76"/>
-      <c r="H36" s="76"/>
+      <c r="D36" s="77"/>
+      <c r="E36" s="77"/>
+      <c r="F36" s="77"/>
+      <c r="G36" s="77"/>
+      <c r="H36" s="77"/>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" s="36" t="s">
@@ -17261,14 +17207,14 @@
       <c r="B37" s="28" t="s">
         <v>1736</v>
       </c>
-      <c r="C37" s="77" t="s">
+      <c r="C37" s="76" t="s">
         <v>1755</v>
       </c>
-      <c r="D37" s="77"/>
-      <c r="E37" s="77"/>
-      <c r="F37" s="77"/>
-      <c r="G37" s="77"/>
-      <c r="H37" s="77"/>
+      <c r="D37" s="76"/>
+      <c r="E37" s="76"/>
+      <c r="F37" s="76"/>
+      <c r="G37" s="76"/>
+      <c r="H37" s="76"/>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" s="36" t="s">
@@ -17277,14 +17223,14 @@
       <c r="B38" s="28" t="s">
         <v>1734</v>
       </c>
-      <c r="C38" s="77" t="s">
+      <c r="C38" s="76" t="s">
         <v>1755</v>
       </c>
-      <c r="D38" s="77"/>
-      <c r="E38" s="77"/>
-      <c r="F38" s="77"/>
-      <c r="G38" s="77"/>
-      <c r="H38" s="77"/>
+      <c r="D38" s="76"/>
+      <c r="E38" s="76"/>
+      <c r="F38" s="76"/>
+      <c r="G38" s="76"/>
+      <c r="H38" s="76"/>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" s="36" t="s">
@@ -17293,14 +17239,14 @@
       <c r="B39" s="28" t="s">
         <v>1734</v>
       </c>
-      <c r="C39" s="76" t="s">
+      <c r="C39" s="77" t="s">
         <v>1753</v>
       </c>
-      <c r="D39" s="76"/>
-      <c r="E39" s="76"/>
-      <c r="F39" s="76"/>
-      <c r="G39" s="76"/>
-      <c r="H39" s="76"/>
+      <c r="D39" s="77"/>
+      <c r="E39" s="77"/>
+      <c r="F39" s="77"/>
+      <c r="G39" s="77"/>
+      <c r="H39" s="77"/>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" s="36" t="s">
@@ -17309,14 +17255,14 @@
       <c r="B40" s="28" t="s">
         <v>1734</v>
       </c>
-      <c r="C40" s="76" t="s">
+      <c r="C40" s="77" t="s">
         <v>1753</v>
       </c>
-      <c r="D40" s="76"/>
-      <c r="E40" s="76"/>
-      <c r="F40" s="76"/>
-      <c r="G40" s="76"/>
-      <c r="H40" s="76"/>
+      <c r="D40" s="77"/>
+      <c r="E40" s="77"/>
+      <c r="F40" s="77"/>
+      <c r="G40" s="77"/>
+      <c r="H40" s="77"/>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" s="36" t="s">
@@ -17325,14 +17271,14 @@
       <c r="B41" s="28" t="s">
         <v>1737</v>
       </c>
-      <c r="C41" s="76" t="s">
+      <c r="C41" s="77" t="s">
         <v>1759</v>
       </c>
-      <c r="D41" s="76"/>
-      <c r="E41" s="76"/>
-      <c r="F41" s="76"/>
-      <c r="G41" s="76"/>
-      <c r="H41" s="76"/>
+      <c r="D41" s="77"/>
+      <c r="E41" s="77"/>
+      <c r="F41" s="77"/>
+      <c r="G41" s="77"/>
+      <c r="H41" s="77"/>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" s="36" t="s">
@@ -17341,14 +17287,14 @@
       <c r="B42" s="28" t="s">
         <v>1738</v>
       </c>
-      <c r="C42" s="76" t="s">
+      <c r="C42" s="77" t="s">
         <v>1761</v>
       </c>
-      <c r="D42" s="76"/>
-      <c r="E42" s="76"/>
-      <c r="F42" s="76"/>
-      <c r="G42" s="76"/>
-      <c r="H42" s="76"/>
+      <c r="D42" s="77"/>
+      <c r="E42" s="77"/>
+      <c r="F42" s="77"/>
+      <c r="G42" s="77"/>
+      <c r="H42" s="77"/>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" s="36" t="s">
@@ -17357,14 +17303,14 @@
       <c r="B43" s="28" t="s">
         <v>1739</v>
       </c>
-      <c r="C43" s="76" t="s">
+      <c r="C43" s="77" t="s">
         <v>1763</v>
       </c>
-      <c r="D43" s="76"/>
-      <c r="E43" s="76"/>
-      <c r="F43" s="76"/>
-      <c r="G43" s="76"/>
-      <c r="H43" s="76"/>
+      <c r="D43" s="77"/>
+      <c r="E43" s="77"/>
+      <c r="F43" s="77"/>
+      <c r="G43" s="77"/>
+      <c r="H43" s="77"/>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" s="36" t="s">
@@ -17373,26 +17319,26 @@
       <c r="B44" s="28" t="s">
         <v>1740</v>
       </c>
-      <c r="C44" s="76" t="s">
+      <c r="C44" s="77" t="s">
         <v>1765</v>
       </c>
-      <c r="D44" s="76"/>
-      <c r="E44" s="76"/>
-      <c r="F44" s="76"/>
-      <c r="G44" s="76"/>
-      <c r="H44" s="76"/>
+      <c r="D44" s="77"/>
+      <c r="E44" s="77"/>
+      <c r="F44" s="77"/>
+      <c r="G44" s="77"/>
+      <c r="H44" s="77"/>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A48" s="75" t="s">
+      <c r="A48" s="78" t="s">
         <v>1754</v>
       </c>
-      <c r="B48" s="75"/>
-      <c r="C48" s="75"/>
-      <c r="D48" s="75"/>
-      <c r="E48" s="75"/>
-      <c r="F48" s="75"/>
-      <c r="G48" s="75"/>
-      <c r="H48" s="75"/>
+      <c r="B48" s="78"/>
+      <c r="C48" s="78"/>
+      <c r="D48" s="78"/>
+      <c r="E48" s="78"/>
+      <c r="F48" s="78"/>
+      <c r="G48" s="78"/>
+      <c r="H48" s="78"/>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
@@ -17405,16 +17351,16 @@
       </c>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A52" s="75" t="s">
+      <c r="A52" s="78" t="s">
         <v>1756</v>
       </c>
-      <c r="B52" s="75"/>
-      <c r="C52" s="75"/>
-      <c r="D52" s="75"/>
-      <c r="E52" s="75"/>
-      <c r="F52" s="75"/>
-      <c r="G52" s="75"/>
-      <c r="H52" s="75"/>
+      <c r="B52" s="78"/>
+      <c r="C52" s="78"/>
+      <c r="D52" s="78"/>
+      <c r="E52" s="78"/>
+      <c r="F52" s="78"/>
+      <c r="G52" s="78"/>
+      <c r="H52" s="78"/>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
@@ -17422,16 +17368,16 @@
       </c>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A57" s="75" t="s">
+      <c r="A57" s="78" t="s">
         <v>1769</v>
       </c>
-      <c r="B57" s="75"/>
-      <c r="C57" s="75"/>
-      <c r="D57" s="75"/>
-      <c r="E57" s="75"/>
-      <c r="F57" s="75"/>
-      <c r="G57" s="75"/>
-      <c r="H57" s="75"/>
+      <c r="B57" s="78"/>
+      <c r="C57" s="78"/>
+      <c r="D57" s="78"/>
+      <c r="E57" s="78"/>
+      <c r="F57" s="78"/>
+      <c r="G57" s="78"/>
+      <c r="H57" s="78"/>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
@@ -17499,12 +17445,12 @@
       </c>
     </row>
     <row r="73" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="H73" s="75" t="s">
+      <c r="H73" s="78" t="s">
         <v>1783</v>
       </c>
-      <c r="I73" s="75"/>
-      <c r="J73" s="75"/>
-      <c r="K73" s="75"/>
+      <c r="I73" s="78"/>
+      <c r="J73" s="78"/>
+      <c r="K73" s="78"/>
     </row>
     <row r="74" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A74" s="55" t="s">
@@ -18071,16 +18017,6 @@
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="C32:H32"/>
-    <mergeCell ref="C33:H33"/>
-    <mergeCell ref="C34:H34"/>
-    <mergeCell ref="C35:H35"/>
-    <mergeCell ref="C36:H36"/>
-    <mergeCell ref="C37:H37"/>
-    <mergeCell ref="C38:H38"/>
-    <mergeCell ref="C39:H39"/>
-    <mergeCell ref="C40:H40"/>
-    <mergeCell ref="C41:H41"/>
     <mergeCell ref="A57:H57"/>
     <mergeCell ref="H73:K73"/>
     <mergeCell ref="C42:H42"/>
@@ -18088,6 +18024,16 @@
     <mergeCell ref="C44:H44"/>
     <mergeCell ref="A48:H48"/>
     <mergeCell ref="A52:H52"/>
+    <mergeCell ref="C37:H37"/>
+    <mergeCell ref="C38:H38"/>
+    <mergeCell ref="C39:H39"/>
+    <mergeCell ref="C40:H40"/>
+    <mergeCell ref="C41:H41"/>
+    <mergeCell ref="C32:H32"/>
+    <mergeCell ref="C33:H33"/>
+    <mergeCell ref="C34:H34"/>
+    <mergeCell ref="C35:H35"/>
+    <mergeCell ref="C36:H36"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78749999999999998" bottom="0.78749999999999998" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -18150,13 +18096,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="75" t="s">
+      <c r="A1" s="78" t="s">
         <v>1905</v>
       </c>
-      <c r="B1" s="75"/>
-      <c r="C1" s="75"/>
-      <c r="D1" s="75"/>
-      <c r="E1" s="75"/>
+      <c r="B1" s="78"/>
+      <c r="C1" s="78"/>
+      <c r="D1" s="78"/>
+      <c r="E1" s="78"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="56" t="s">

</xml_diff>

<commit_message>
Palette 59: colours 12/13 blue-green accents, copies of the stone walls (193-200) and overlays (151-155) without 12/13, green mosaic in the S'Riel hall
</commit_message>
<xml_diff>
--- a/AmbermoonAdvanced.xlsx
+++ b/AmbermoonAdvanced.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Robert\source\repos\Ambermoon-Advanced\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E14F54B-0700-4FE1-A2FA-2CA5868C6A49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2B8030B-FB99-4B6A-B152-536B6244491A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" firstSheet="36" activeTab="42" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -78,7 +78,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3181" uniqueCount="2289">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3220" uniqueCount="2303">
   <si>
     <t>Map texts</t>
   </si>
@@ -7061,7 +7061,49 @@
     <t>Temple rework pilot, only reachable with the cheat map jump (t, 487) or the remake teleport cheat. Built by assets/Temples/tools/build_prototype.py. Labdata 46, palette 59, music 22 (later 33). Exit to 520 (37,41) like 444. Reuses chests 116/117 of map 444.</t>
   </si>
   <si>
-    <t>Temple base (first used by the S'Riel prototype, map 487): copy of labdata 5 (Gala temple) with floor 20, ceiling 8, new walls 131-134 (wall 99 with column frames 24/25 and rosette 71 / window 72 / crest 74) and object group 40 (serpent totem, texture 28). With palette 59 'Wüstentempel' (stone colours as sandstone, same index meaning as palette 6) everything turns into sandstone. Details: assets/Temples/Labdata 46.md</t>
+    <t>Copy of wall 96 (Prunktür) without the colours 12/13 (replaced by 3/5), for palette 59 where 12/13 are blue-green accents</t>
+  </si>
+  <si>
+    <t>Labdata 46 (temple base)</t>
+  </si>
+  <si>
+    <t>Copy of wall 98 (Doppelbogen) without the colours 12/13 (replaced by 3/5), for palette 59 where 12/13 are blue-green accents</t>
+  </si>
+  <si>
+    <t>Copy of wall 99 (Grundwand) without the colours 12/13 (replaced by 3/5), for palette 59 where 12/13 are blue-green accents</t>
+  </si>
+  <si>
+    <t>Copy of wall 100 (Reliefpfeiler) without the colours 12/13 (replaced by 3/5), for palette 59 where 12/13 are blue-green accents</t>
+  </si>
+  <si>
+    <t>Copy of wall 103 (Relieffries) without the colours 12/13 (replaced by 3/5), for palette 59 where 12/13 are blue-green accents</t>
+  </si>
+  <si>
+    <t>Copy of wall 104 (Dunkles Tor im Relief) without the colours 12/13 (replaced by 3/5), for palette 59 where 12/13 are blue-green accents</t>
+  </si>
+  <si>
+    <t>Copy of wall 125 (Treppe hoch) without the colours 12/13 (replaced by 3/5), for palette 59 where 12/13 are blue-green accents</t>
+  </si>
+  <si>
+    <t>Copy of wall 126 (Treppe runter) without the colours 12/13 (replaced by 3/5), for palette 59 where 12/13 are blue-green accents</t>
+  </si>
+  <si>
+    <t>Copy of overlay 24 (Pillar frame left) without the colours 12/13 (replaced by 3/5)</t>
+  </si>
+  <si>
+    <t>Copy of overlay 25 (Pillar frame right) without the colours 12/13 (replaced by 3/5)</t>
+  </si>
+  <si>
+    <t>Copy of overlay 39 (Stone head) without the colours 12/13 (replaced by 3/5)</t>
+  </si>
+  <si>
+    <t>Copy of overlay 96 (Door pillar frame left) without the colours 12/13 (replaced by 3/5)</t>
+  </si>
+  <si>
+    <t>Copy of overlay 97 (Door pillar frame right) without the colours 12/13 (replaced by 3/5)</t>
+  </si>
+  <si>
+    <t>Temple base (first used by the S'Riel prototype, map 487): copy of labdata 5 (Gala temple) with floor 20, ceiling 8, new walls 131-134 (wall 99 with column frames and rosette / window / crest) and object group 40 (serpent totem). The stone walls and overlays point to copies without the colours 12/13 (walls 193-200, overlays 151-155), so in palette 59 'Wüstentempel' the walls are sandstone and 12/13 are blue-green accents (glass, mosaics, marble, books). Details: assets/Temples/Labdata 46.md</t>
   </si>
 </sst>
 </file>
@@ -7707,17 +7749,17 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="27" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="21" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="27" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="21" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -10176,7 +10218,7 @@
         <v>46</v>
       </c>
       <c r="B14" t="s">
-        <v>2288</v>
+        <v>2302</v>
       </c>
     </row>
   </sheetData>
@@ -14662,7 +14704,7 @@
 
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1500-000000000000}">
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:D29"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="67.85546875" customWidth="1"/>
@@ -14960,6 +15002,118 @@
         <v>1520</v>
       </c>
       <c r="D21" t="s">
+        <v>1530</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>193</v>
+      </c>
+      <c r="B22" t="s">
+        <v>2288</v>
+      </c>
+      <c r="C22" t="s">
+        <v>2289</v>
+      </c>
+      <c r="D22" t="s">
+        <v>1530</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>194</v>
+      </c>
+      <c r="B23" t="s">
+        <v>2290</v>
+      </c>
+      <c r="C23" t="s">
+        <v>2289</v>
+      </c>
+      <c r="D23" t="s">
+        <v>1530</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>195</v>
+      </c>
+      <c r="B24" t="s">
+        <v>2291</v>
+      </c>
+      <c r="C24" t="s">
+        <v>2289</v>
+      </c>
+      <c r="D24" t="s">
+        <v>1530</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>196</v>
+      </c>
+      <c r="B25" t="s">
+        <v>2292</v>
+      </c>
+      <c r="C25" t="s">
+        <v>2289</v>
+      </c>
+      <c r="D25" t="s">
+        <v>1530</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>197</v>
+      </c>
+      <c r="B26" t="s">
+        <v>2293</v>
+      </c>
+      <c r="C26" t="s">
+        <v>2289</v>
+      </c>
+      <c r="D26" t="s">
+        <v>1530</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>198</v>
+      </c>
+      <c r="B27" t="s">
+        <v>2294</v>
+      </c>
+      <c r="C27" t="s">
+        <v>2289</v>
+      </c>
+      <c r="D27" t="s">
+        <v>1530</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A28">
+        <v>199</v>
+      </c>
+      <c r="B28" t="s">
+        <v>2295</v>
+      </c>
+      <c r="C28" t="s">
+        <v>2289</v>
+      </c>
+      <c r="D28" t="s">
+        <v>1530</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A29">
+        <v>200</v>
+      </c>
+      <c r="B29" t="s">
+        <v>2296</v>
+      </c>
+      <c r="C29" t="s">
+        <v>2289</v>
+      </c>
+      <c r="D29" t="s">
         <v>1530</v>
       </c>
     </row>
@@ -14975,7 +15129,7 @@
 
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1600-000000000000}">
-  <dimension ref="A1:E60"/>
+  <dimension ref="A1:E65"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="43.7109375" customWidth="1"/>
@@ -15824,6 +15978,76 @@
       </c>
       <c r="D60" t="s">
         <v>2143</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A61">
+        <v>151</v>
+      </c>
+      <c r="B61" t="s">
+        <v>2297</v>
+      </c>
+      <c r="C61" t="s">
+        <v>2289</v>
+      </c>
+      <c r="D61" t="s">
+        <v>1558</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A62">
+        <v>152</v>
+      </c>
+      <c r="B62" t="s">
+        <v>2298</v>
+      </c>
+      <c r="C62" t="s">
+        <v>2289</v>
+      </c>
+      <c r="D62" t="s">
+        <v>1558</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A63">
+        <v>153</v>
+      </c>
+      <c r="B63" t="s">
+        <v>2299</v>
+      </c>
+      <c r="C63" t="s">
+        <v>2289</v>
+      </c>
+      <c r="D63" t="s">
+        <v>1558</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A64">
+        <v>154</v>
+      </c>
+      <c r="B64" t="s">
+        <v>2300</v>
+      </c>
+      <c r="C64" t="s">
+        <v>2289</v>
+      </c>
+      <c r="D64" t="s">
+        <v>1558</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A65">
+        <v>155</v>
+      </c>
+      <c r="B65" t="s">
+        <v>2301</v>
+      </c>
+      <c r="C65" t="s">
+        <v>2289</v>
+      </c>
+      <c r="D65" t="s">
+        <v>1558</v>
       </c>
     </row>
   </sheetData>
@@ -17127,14 +17351,14 @@
       <c r="B32" s="54" t="s">
         <v>1745</v>
       </c>
-      <c r="C32" s="75" t="s">
+      <c r="C32" s="78" t="s">
         <v>1746</v>
       </c>
-      <c r="D32" s="75"/>
-      <c r="E32" s="75"/>
-      <c r="F32" s="75"/>
-      <c r="G32" s="75"/>
-      <c r="H32" s="75"/>
+      <c r="D32" s="78"/>
+      <c r="E32" s="78"/>
+      <c r="F32" s="78"/>
+      <c r="G32" s="78"/>
+      <c r="H32" s="78"/>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" s="36" t="s">
@@ -17143,14 +17367,14 @@
       <c r="B33" s="28" t="s">
         <v>1748</v>
       </c>
-      <c r="C33" s="76" t="s">
+      <c r="C33" s="77" t="s">
         <v>1749</v>
       </c>
-      <c r="D33" s="76"/>
-      <c r="E33" s="76"/>
-      <c r="F33" s="76"/>
-      <c r="G33" s="76"/>
-      <c r="H33" s="76"/>
+      <c r="D33" s="77"/>
+      <c r="E33" s="77"/>
+      <c r="F33" s="77"/>
+      <c r="G33" s="77"/>
+      <c r="H33" s="77"/>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" s="36" t="s">
@@ -17159,14 +17383,14 @@
       <c r="B34" s="28" t="s">
         <v>1748</v>
       </c>
-      <c r="C34" s="76" t="s">
+      <c r="C34" s="77" t="s">
         <v>1749</v>
       </c>
-      <c r="D34" s="76"/>
-      <c r="E34" s="76"/>
-      <c r="F34" s="76"/>
-      <c r="G34" s="76"/>
-      <c r="H34" s="76"/>
+      <c r="D34" s="77"/>
+      <c r="E34" s="77"/>
+      <c r="F34" s="77"/>
+      <c r="G34" s="77"/>
+      <c r="H34" s="77"/>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" s="36" t="s">
@@ -17175,14 +17399,14 @@
       <c r="B35" s="28" t="s">
         <v>1748</v>
       </c>
-      <c r="C35" s="76" t="s">
+      <c r="C35" s="77" t="s">
         <v>1749</v>
       </c>
-      <c r="D35" s="76"/>
-      <c r="E35" s="76"/>
-      <c r="F35" s="76"/>
-      <c r="G35" s="76"/>
-      <c r="H35" s="76"/>
+      <c r="D35" s="77"/>
+      <c r="E35" s="77"/>
+      <c r="F35" s="77"/>
+      <c r="G35" s="77"/>
+      <c r="H35" s="77"/>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" s="36" t="s">
@@ -17191,14 +17415,14 @@
       <c r="B36" s="28" t="s">
         <v>1734</v>
       </c>
-      <c r="C36" s="77" t="s">
+      <c r="C36" s="76" t="s">
         <v>1753</v>
       </c>
-      <c r="D36" s="77"/>
-      <c r="E36" s="77"/>
-      <c r="F36" s="77"/>
-      <c r="G36" s="77"/>
-      <c r="H36" s="77"/>
+      <c r="D36" s="76"/>
+      <c r="E36" s="76"/>
+      <c r="F36" s="76"/>
+      <c r="G36" s="76"/>
+      <c r="H36" s="76"/>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" s="36" t="s">
@@ -17207,14 +17431,14 @@
       <c r="B37" s="28" t="s">
         <v>1736</v>
       </c>
-      <c r="C37" s="76" t="s">
+      <c r="C37" s="77" t="s">
         <v>1755</v>
       </c>
-      <c r="D37" s="76"/>
-      <c r="E37" s="76"/>
-      <c r="F37" s="76"/>
-      <c r="G37" s="76"/>
-      <c r="H37" s="76"/>
+      <c r="D37" s="77"/>
+      <c r="E37" s="77"/>
+      <c r="F37" s="77"/>
+      <c r="G37" s="77"/>
+      <c r="H37" s="77"/>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" s="36" t="s">
@@ -17223,14 +17447,14 @@
       <c r="B38" s="28" t="s">
         <v>1734</v>
       </c>
-      <c r="C38" s="76" t="s">
+      <c r="C38" s="77" t="s">
         <v>1755</v>
       </c>
-      <c r="D38" s="76"/>
-      <c r="E38" s="76"/>
-      <c r="F38" s="76"/>
-      <c r="G38" s="76"/>
-      <c r="H38" s="76"/>
+      <c r="D38" s="77"/>
+      <c r="E38" s="77"/>
+      <c r="F38" s="77"/>
+      <c r="G38" s="77"/>
+      <c r="H38" s="77"/>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" s="36" t="s">
@@ -17239,14 +17463,14 @@
       <c r="B39" s="28" t="s">
         <v>1734</v>
       </c>
-      <c r="C39" s="77" t="s">
+      <c r="C39" s="76" t="s">
         <v>1753</v>
       </c>
-      <c r="D39" s="77"/>
-      <c r="E39" s="77"/>
-      <c r="F39" s="77"/>
-      <c r="G39" s="77"/>
-      <c r="H39" s="77"/>
+      <c r="D39" s="76"/>
+      <c r="E39" s="76"/>
+      <c r="F39" s="76"/>
+      <c r="G39" s="76"/>
+      <c r="H39" s="76"/>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" s="36" t="s">
@@ -17255,14 +17479,14 @@
       <c r="B40" s="28" t="s">
         <v>1734</v>
       </c>
-      <c r="C40" s="77" t="s">
+      <c r="C40" s="76" t="s">
         <v>1753</v>
       </c>
-      <c r="D40" s="77"/>
-      <c r="E40" s="77"/>
-      <c r="F40" s="77"/>
-      <c r="G40" s="77"/>
-      <c r="H40" s="77"/>
+      <c r="D40" s="76"/>
+      <c r="E40" s="76"/>
+      <c r="F40" s="76"/>
+      <c r="G40" s="76"/>
+      <c r="H40" s="76"/>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" s="36" t="s">
@@ -17271,14 +17495,14 @@
       <c r="B41" s="28" t="s">
         <v>1737</v>
       </c>
-      <c r="C41" s="77" t="s">
+      <c r="C41" s="76" t="s">
         <v>1759</v>
       </c>
-      <c r="D41" s="77"/>
-      <c r="E41" s="77"/>
-      <c r="F41" s="77"/>
-      <c r="G41" s="77"/>
-      <c r="H41" s="77"/>
+      <c r="D41" s="76"/>
+      <c r="E41" s="76"/>
+      <c r="F41" s="76"/>
+      <c r="G41" s="76"/>
+      <c r="H41" s="76"/>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" s="36" t="s">
@@ -17287,14 +17511,14 @@
       <c r="B42" s="28" t="s">
         <v>1738</v>
       </c>
-      <c r="C42" s="77" t="s">
+      <c r="C42" s="76" t="s">
         <v>1761</v>
       </c>
-      <c r="D42" s="77"/>
-      <c r="E42" s="77"/>
-      <c r="F42" s="77"/>
-      <c r="G42" s="77"/>
-      <c r="H42" s="77"/>
+      <c r="D42" s="76"/>
+      <c r="E42" s="76"/>
+      <c r="F42" s="76"/>
+      <c r="G42" s="76"/>
+      <c r="H42" s="76"/>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" s="36" t="s">
@@ -17303,14 +17527,14 @@
       <c r="B43" s="28" t="s">
         <v>1739</v>
       </c>
-      <c r="C43" s="77" t="s">
+      <c r="C43" s="76" t="s">
         <v>1763</v>
       </c>
-      <c r="D43" s="77"/>
-      <c r="E43" s="77"/>
-      <c r="F43" s="77"/>
-      <c r="G43" s="77"/>
-      <c r="H43" s="77"/>
+      <c r="D43" s="76"/>
+      <c r="E43" s="76"/>
+      <c r="F43" s="76"/>
+      <c r="G43" s="76"/>
+      <c r="H43" s="76"/>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" s="36" t="s">
@@ -17319,26 +17543,26 @@
       <c r="B44" s="28" t="s">
         <v>1740</v>
       </c>
-      <c r="C44" s="77" t="s">
+      <c r="C44" s="76" t="s">
         <v>1765</v>
       </c>
-      <c r="D44" s="77"/>
-      <c r="E44" s="77"/>
-      <c r="F44" s="77"/>
-      <c r="G44" s="77"/>
-      <c r="H44" s="77"/>
+      <c r="D44" s="76"/>
+      <c r="E44" s="76"/>
+      <c r="F44" s="76"/>
+      <c r="G44" s="76"/>
+      <c r="H44" s="76"/>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A48" s="78" t="s">
+      <c r="A48" s="75" t="s">
         <v>1754</v>
       </c>
-      <c r="B48" s="78"/>
-      <c r="C48" s="78"/>
-      <c r="D48" s="78"/>
-      <c r="E48" s="78"/>
-      <c r="F48" s="78"/>
-      <c r="G48" s="78"/>
-      <c r="H48" s="78"/>
+      <c r="B48" s="75"/>
+      <c r="C48" s="75"/>
+      <c r="D48" s="75"/>
+      <c r="E48" s="75"/>
+      <c r="F48" s="75"/>
+      <c r="G48" s="75"/>
+      <c r="H48" s="75"/>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
@@ -17351,16 +17575,16 @@
       </c>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A52" s="78" t="s">
+      <c r="A52" s="75" t="s">
         <v>1756</v>
       </c>
-      <c r="B52" s="78"/>
-      <c r="C52" s="78"/>
-      <c r="D52" s="78"/>
-      <c r="E52" s="78"/>
-      <c r="F52" s="78"/>
-      <c r="G52" s="78"/>
-      <c r="H52" s="78"/>
+      <c r="B52" s="75"/>
+      <c r="C52" s="75"/>
+      <c r="D52" s="75"/>
+      <c r="E52" s="75"/>
+      <c r="F52" s="75"/>
+      <c r="G52" s="75"/>
+      <c r="H52" s="75"/>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
@@ -17368,16 +17592,16 @@
       </c>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A57" s="78" t="s">
+      <c r="A57" s="75" t="s">
         <v>1769</v>
       </c>
-      <c r="B57" s="78"/>
-      <c r="C57" s="78"/>
-      <c r="D57" s="78"/>
-      <c r="E57" s="78"/>
-      <c r="F57" s="78"/>
-      <c r="G57" s="78"/>
-      <c r="H57" s="78"/>
+      <c r="B57" s="75"/>
+      <c r="C57" s="75"/>
+      <c r="D57" s="75"/>
+      <c r="E57" s="75"/>
+      <c r="F57" s="75"/>
+      <c r="G57" s="75"/>
+      <c r="H57" s="75"/>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
@@ -17445,12 +17669,12 @@
       </c>
     </row>
     <row r="73" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="H73" s="78" t="s">
+      <c r="H73" s="75" t="s">
         <v>1783</v>
       </c>
-      <c r="I73" s="78"/>
-      <c r="J73" s="78"/>
-      <c r="K73" s="78"/>
+      <c r="I73" s="75"/>
+      <c r="J73" s="75"/>
+      <c r="K73" s="75"/>
     </row>
     <row r="74" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A74" s="55" t="s">
@@ -18017,6 +18241,16 @@
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="C32:H32"/>
+    <mergeCell ref="C33:H33"/>
+    <mergeCell ref="C34:H34"/>
+    <mergeCell ref="C35:H35"/>
+    <mergeCell ref="C36:H36"/>
+    <mergeCell ref="C37:H37"/>
+    <mergeCell ref="C38:H38"/>
+    <mergeCell ref="C39:H39"/>
+    <mergeCell ref="C40:H40"/>
+    <mergeCell ref="C41:H41"/>
     <mergeCell ref="A57:H57"/>
     <mergeCell ref="H73:K73"/>
     <mergeCell ref="C42:H42"/>
@@ -18024,16 +18258,6 @@
     <mergeCell ref="C44:H44"/>
     <mergeCell ref="A48:H48"/>
     <mergeCell ref="A52:H52"/>
-    <mergeCell ref="C37:H37"/>
-    <mergeCell ref="C38:H38"/>
-    <mergeCell ref="C39:H39"/>
-    <mergeCell ref="C40:H40"/>
-    <mergeCell ref="C41:H41"/>
-    <mergeCell ref="C32:H32"/>
-    <mergeCell ref="C33:H33"/>
-    <mergeCell ref="C34:H34"/>
-    <mergeCell ref="C35:H35"/>
-    <mergeCell ref="C36:H36"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78749999999999998" bottom="0.78749999999999998" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -18096,13 +18320,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="78" t="s">
+      <c r="A1" s="75" t="s">
         <v>1905</v>
       </c>
-      <c r="B1" s="78"/>
-      <c r="C1" s="78"/>
-      <c r="D1" s="78"/>
-      <c r="E1" s="78"/>
+      <c r="B1" s="75"/>
+      <c r="C1" s="75"/>
+      <c r="D1" s="75"/>
+      <c r="E1" s="75"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="56" t="s">

</xml_diff>

<commit_message>
Temple prototype S'Orel (map 488): outer corridor with guards and spike trap, gate with key 388, armoury and training hall, palette 60, monster group 172
</commit_message>
<xml_diff>
--- a/AmbermoonAdvanced.xlsx
+++ b/AmbermoonAdvanced.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Robert\source\repos\Ambermoon-Advanced\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2B8030B-FB99-4B6A-B152-536B6244491A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1B19C78-2B21-40A6-B758-69FAA40B6061}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" firstSheet="36" activeTab="42" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -78,7 +78,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3220" uniqueCount="2303">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3223" uniqueCount="2305">
   <si>
     <t>Map texts</t>
   </si>
@@ -7104,6 +7104,12 @@
   </si>
   <si>
     <t>Temple base (first used by the S'Riel prototype, map 487): copy of labdata 5 (Gala temple) with floor 20, ceiling 8, new walls 131-134 (wall 99 with column frames and rosette / window / crest) and object group 40 (serpent totem). The stone walls and overlays point to copies without the colours 12/13 (walls 193-200, overlays 151-155), so in palette 59 'Wüstentempel' the walls are sandstone and 12/13 are blue-green accents (glass, mosaics, marble, books). Details: assets/Temples/Labdata 46.md</t>
+  </si>
+  <si>
+    <t>Palast des S'Orel (Prototyp) / Palace of S'Orel (prototype)</t>
+  </si>
+  <si>
+    <t>Temple rework S'Orel (barracks), only reachable with the cheat map jump (t, 488) or the remake teleport cheat. Built by assets/Temples/tools/build_prototype.py. Labdata 46, palette 60 'Kaserne', music 18, no map. New monster group 172 (6 magic guards). Reuses door 33 (key 388) and chests 118/119 of map 445. Exit to 525 (33,28) like 445.</t>
   </si>
 </sst>
 </file>
@@ -7749,17 +7755,17 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="21" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="27" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="27" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="21" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -9354,7 +9360,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
-  <dimension ref="A1:D48"/>
+  <dimension ref="A1:D49"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7.7109375" customWidth="1"/>
@@ -10002,6 +10008,20 @@
       </c>
       <c r="D48" t="s">
         <v>2287</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A49">
+        <v>488</v>
+      </c>
+      <c r="B49" t="s">
+        <v>2303</v>
+      </c>
+      <c r="C49" t="s">
+        <v>911</v>
+      </c>
+      <c r="D49" t="s">
+        <v>2304</v>
       </c>
     </row>
   </sheetData>
@@ -17351,14 +17371,14 @@
       <c r="B32" s="54" t="s">
         <v>1745</v>
       </c>
-      <c r="C32" s="78" t="s">
+      <c r="C32" s="75" t="s">
         <v>1746</v>
       </c>
-      <c r="D32" s="78"/>
-      <c r="E32" s="78"/>
-      <c r="F32" s="78"/>
-      <c r="G32" s="78"/>
-      <c r="H32" s="78"/>
+      <c r="D32" s="75"/>
+      <c r="E32" s="75"/>
+      <c r="F32" s="75"/>
+      <c r="G32" s="75"/>
+      <c r="H32" s="75"/>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" s="36" t="s">
@@ -17367,14 +17387,14 @@
       <c r="B33" s="28" t="s">
         <v>1748</v>
       </c>
-      <c r="C33" s="77" t="s">
+      <c r="C33" s="76" t="s">
         <v>1749</v>
       </c>
-      <c r="D33" s="77"/>
-      <c r="E33" s="77"/>
-      <c r="F33" s="77"/>
-      <c r="G33" s="77"/>
-      <c r="H33" s="77"/>
+      <c r="D33" s="76"/>
+      <c r="E33" s="76"/>
+      <c r="F33" s="76"/>
+      <c r="G33" s="76"/>
+      <c r="H33" s="76"/>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" s="36" t="s">
@@ -17383,14 +17403,14 @@
       <c r="B34" s="28" t="s">
         <v>1748</v>
       </c>
-      <c r="C34" s="77" t="s">
+      <c r="C34" s="76" t="s">
         <v>1749</v>
       </c>
-      <c r="D34" s="77"/>
-      <c r="E34" s="77"/>
-      <c r="F34" s="77"/>
-      <c r="G34" s="77"/>
-      <c r="H34" s="77"/>
+      <c r="D34" s="76"/>
+      <c r="E34" s="76"/>
+      <c r="F34" s="76"/>
+      <c r="G34" s="76"/>
+      <c r="H34" s="76"/>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" s="36" t="s">
@@ -17399,14 +17419,14 @@
       <c r="B35" s="28" t="s">
         <v>1748</v>
       </c>
-      <c r="C35" s="77" t="s">
+      <c r="C35" s="76" t="s">
         <v>1749</v>
       </c>
-      <c r="D35" s="77"/>
-      <c r="E35" s="77"/>
-      <c r="F35" s="77"/>
-      <c r="G35" s="77"/>
-      <c r="H35" s="77"/>
+      <c r="D35" s="76"/>
+      <c r="E35" s="76"/>
+      <c r="F35" s="76"/>
+      <c r="G35" s="76"/>
+      <c r="H35" s="76"/>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" s="36" t="s">
@@ -17415,14 +17435,14 @@
       <c r="B36" s="28" t="s">
         <v>1734</v>
       </c>
-      <c r="C36" s="76" t="s">
+      <c r="C36" s="77" t="s">
         <v>1753</v>
       </c>
-      <c r="D36" s="76"/>
-      <c r="E36" s="76"/>
-      <c r="F36" s="76"/>
-      <c r="G36" s="76"/>
-      <c r="H36" s="76"/>
+      <c r="D36" s="77"/>
+      <c r="E36" s="77"/>
+      <c r="F36" s="77"/>
+      <c r="G36" s="77"/>
+      <c r="H36" s="77"/>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" s="36" t="s">
@@ -17431,14 +17451,14 @@
       <c r="B37" s="28" t="s">
         <v>1736</v>
       </c>
-      <c r="C37" s="77" t="s">
+      <c r="C37" s="76" t="s">
         <v>1755</v>
       </c>
-      <c r="D37" s="77"/>
-      <c r="E37" s="77"/>
-      <c r="F37" s="77"/>
-      <c r="G37" s="77"/>
-      <c r="H37" s="77"/>
+      <c r="D37" s="76"/>
+      <c r="E37" s="76"/>
+      <c r="F37" s="76"/>
+      <c r="G37" s="76"/>
+      <c r="H37" s="76"/>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" s="36" t="s">
@@ -17447,14 +17467,14 @@
       <c r="B38" s="28" t="s">
         <v>1734</v>
       </c>
-      <c r="C38" s="77" t="s">
+      <c r="C38" s="76" t="s">
         <v>1755</v>
       </c>
-      <c r="D38" s="77"/>
-      <c r="E38" s="77"/>
-      <c r="F38" s="77"/>
-      <c r="G38" s="77"/>
-      <c r="H38" s="77"/>
+      <c r="D38" s="76"/>
+      <c r="E38" s="76"/>
+      <c r="F38" s="76"/>
+      <c r="G38" s="76"/>
+      <c r="H38" s="76"/>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" s="36" t="s">
@@ -17463,14 +17483,14 @@
       <c r="B39" s="28" t="s">
         <v>1734</v>
       </c>
-      <c r="C39" s="76" t="s">
+      <c r="C39" s="77" t="s">
         <v>1753</v>
       </c>
-      <c r="D39" s="76"/>
-      <c r="E39" s="76"/>
-      <c r="F39" s="76"/>
-      <c r="G39" s="76"/>
-      <c r="H39" s="76"/>
+      <c r="D39" s="77"/>
+      <c r="E39" s="77"/>
+      <c r="F39" s="77"/>
+      <c r="G39" s="77"/>
+      <c r="H39" s="77"/>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" s="36" t="s">
@@ -17479,14 +17499,14 @@
       <c r="B40" s="28" t="s">
         <v>1734</v>
       </c>
-      <c r="C40" s="76" t="s">
+      <c r="C40" s="77" t="s">
         <v>1753</v>
       </c>
-      <c r="D40" s="76"/>
-      <c r="E40" s="76"/>
-      <c r="F40" s="76"/>
-      <c r="G40" s="76"/>
-      <c r="H40" s="76"/>
+      <c r="D40" s="77"/>
+      <c r="E40" s="77"/>
+      <c r="F40" s="77"/>
+      <c r="G40" s="77"/>
+      <c r="H40" s="77"/>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" s="36" t="s">
@@ -17495,14 +17515,14 @@
       <c r="B41" s="28" t="s">
         <v>1737</v>
       </c>
-      <c r="C41" s="76" t="s">
+      <c r="C41" s="77" t="s">
         <v>1759</v>
       </c>
-      <c r="D41" s="76"/>
-      <c r="E41" s="76"/>
-      <c r="F41" s="76"/>
-      <c r="G41" s="76"/>
-      <c r="H41" s="76"/>
+      <c r="D41" s="77"/>
+      <c r="E41" s="77"/>
+      <c r="F41" s="77"/>
+      <c r="G41" s="77"/>
+      <c r="H41" s="77"/>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" s="36" t="s">
@@ -17511,14 +17531,14 @@
       <c r="B42" s="28" t="s">
         <v>1738</v>
       </c>
-      <c r="C42" s="76" t="s">
+      <c r="C42" s="77" t="s">
         <v>1761</v>
       </c>
-      <c r="D42" s="76"/>
-      <c r="E42" s="76"/>
-      <c r="F42" s="76"/>
-      <c r="G42" s="76"/>
-      <c r="H42" s="76"/>
+      <c r="D42" s="77"/>
+      <c r="E42" s="77"/>
+      <c r="F42" s="77"/>
+      <c r="G42" s="77"/>
+      <c r="H42" s="77"/>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" s="36" t="s">
@@ -17527,14 +17547,14 @@
       <c r="B43" s="28" t="s">
         <v>1739</v>
       </c>
-      <c r="C43" s="76" t="s">
+      <c r="C43" s="77" t="s">
         <v>1763</v>
       </c>
-      <c r="D43" s="76"/>
-      <c r="E43" s="76"/>
-      <c r="F43" s="76"/>
-      <c r="G43" s="76"/>
-      <c r="H43" s="76"/>
+      <c r="D43" s="77"/>
+      <c r="E43" s="77"/>
+      <c r="F43" s="77"/>
+      <c r="G43" s="77"/>
+      <c r="H43" s="77"/>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" s="36" t="s">
@@ -17543,26 +17563,26 @@
       <c r="B44" s="28" t="s">
         <v>1740</v>
       </c>
-      <c r="C44" s="76" t="s">
+      <c r="C44" s="77" t="s">
         <v>1765</v>
       </c>
-      <c r="D44" s="76"/>
-      <c r="E44" s="76"/>
-      <c r="F44" s="76"/>
-      <c r="G44" s="76"/>
-      <c r="H44" s="76"/>
+      <c r="D44" s="77"/>
+      <c r="E44" s="77"/>
+      <c r="F44" s="77"/>
+      <c r="G44" s="77"/>
+      <c r="H44" s="77"/>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A48" s="75" t="s">
+      <c r="A48" s="78" t="s">
         <v>1754</v>
       </c>
-      <c r="B48" s="75"/>
-      <c r="C48" s="75"/>
-      <c r="D48" s="75"/>
-      <c r="E48" s="75"/>
-      <c r="F48" s="75"/>
-      <c r="G48" s="75"/>
-      <c r="H48" s="75"/>
+      <c r="B48" s="78"/>
+      <c r="C48" s="78"/>
+      <c r="D48" s="78"/>
+      <c r="E48" s="78"/>
+      <c r="F48" s="78"/>
+      <c r="G48" s="78"/>
+      <c r="H48" s="78"/>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
@@ -17575,16 +17595,16 @@
       </c>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A52" s="75" t="s">
+      <c r="A52" s="78" t="s">
         <v>1756</v>
       </c>
-      <c r="B52" s="75"/>
-      <c r="C52" s="75"/>
-      <c r="D52" s="75"/>
-      <c r="E52" s="75"/>
-      <c r="F52" s="75"/>
-      <c r="G52" s="75"/>
-      <c r="H52" s="75"/>
+      <c r="B52" s="78"/>
+      <c r="C52" s="78"/>
+      <c r="D52" s="78"/>
+      <c r="E52" s="78"/>
+      <c r="F52" s="78"/>
+      <c r="G52" s="78"/>
+      <c r="H52" s="78"/>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
@@ -17592,16 +17612,16 @@
       </c>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A57" s="75" t="s">
+      <c r="A57" s="78" t="s">
         <v>1769</v>
       </c>
-      <c r="B57" s="75"/>
-      <c r="C57" s="75"/>
-      <c r="D57" s="75"/>
-      <c r="E57" s="75"/>
-      <c r="F57" s="75"/>
-      <c r="G57" s="75"/>
-      <c r="H57" s="75"/>
+      <c r="B57" s="78"/>
+      <c r="C57" s="78"/>
+      <c r="D57" s="78"/>
+      <c r="E57" s="78"/>
+      <c r="F57" s="78"/>
+      <c r="G57" s="78"/>
+      <c r="H57" s="78"/>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
@@ -17669,12 +17689,12 @@
       </c>
     </row>
     <row r="73" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="H73" s="75" t="s">
+      <c r="H73" s="78" t="s">
         <v>1783</v>
       </c>
-      <c r="I73" s="75"/>
-      <c r="J73" s="75"/>
-      <c r="K73" s="75"/>
+      <c r="I73" s="78"/>
+      <c r="J73" s="78"/>
+      <c r="K73" s="78"/>
     </row>
     <row r="74" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A74" s="55" t="s">
@@ -18241,16 +18261,6 @@
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="C32:H32"/>
-    <mergeCell ref="C33:H33"/>
-    <mergeCell ref="C34:H34"/>
-    <mergeCell ref="C35:H35"/>
-    <mergeCell ref="C36:H36"/>
-    <mergeCell ref="C37:H37"/>
-    <mergeCell ref="C38:H38"/>
-    <mergeCell ref="C39:H39"/>
-    <mergeCell ref="C40:H40"/>
-    <mergeCell ref="C41:H41"/>
     <mergeCell ref="A57:H57"/>
     <mergeCell ref="H73:K73"/>
     <mergeCell ref="C42:H42"/>
@@ -18258,6 +18268,16 @@
     <mergeCell ref="C44:H44"/>
     <mergeCell ref="A48:H48"/>
     <mergeCell ref="A52:H52"/>
+    <mergeCell ref="C37:H37"/>
+    <mergeCell ref="C38:H38"/>
+    <mergeCell ref="C39:H39"/>
+    <mergeCell ref="C40:H40"/>
+    <mergeCell ref="C41:H41"/>
+    <mergeCell ref="C32:H32"/>
+    <mergeCell ref="C33:H33"/>
+    <mergeCell ref="C34:H34"/>
+    <mergeCell ref="C35:H35"/>
+    <mergeCell ref="C36:H36"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78749999999999998" bottom="0.78749999999999998" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -18320,13 +18340,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="75" t="s">
+      <c r="A1" s="78" t="s">
         <v>1905</v>
       </c>
-      <c r="B1" s="75"/>
-      <c r="C1" s="75"/>
-      <c r="D1" s="75"/>
-      <c r="E1" s="75"/>
+      <c r="B1" s="78"/>
+      <c r="C1" s="78"/>
+      <c r="D1" s="78"/>
+      <c r="E1" s="78"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="56" t="s">

</xml_diff>

<commit_message>
Savegame patching note: automap 488
</commit_message>
<xml_diff>
--- a/AmbermoonAdvanced.xlsx
+++ b/AmbermoonAdvanced.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Robert\source\repos\Ambermoon-Advanced\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1B19C78-2B21-40A6-B758-69FAA40B6061}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B51921E-0CD2-4DBC-9081-07E7CC7B47CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" firstSheet="36" activeTab="42" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7049,9 +7049,6 @@
     <t>Palast des S'Riel (Prototyp) / Palace of S'Riel (prototype)</t>
   </si>
   <si>
-    <t>Add automaps 485 (27x27, 92 bytes), 486 (11x19, 27 bytes) and 487 (17x17, 37 bytes). They were missing in Save.00, entering 485/486 on the Amiga ends in a fatal error (Init_automap loads the entry for every 3D map).</t>
-  </si>
-  <si>
     <t>Chosen as temple music, not in Music.amb yet</t>
   </si>
   <si>
@@ -7110,6 +7107,9 @@
   </si>
   <si>
     <t>Temple rework S'Orel (barracks), only reachable with the cheat map jump (t, 488) or the remake teleport cheat. Built by assets/Temples/tools/build_prototype.py. Labdata 46, palette 60 'Kaserne', music 18, no map. New monster group 172 (6 magic guards). Reuses door 33 (key 388) and chests 118/119 of map 445. Exit to 525 (33,28) like 445.</t>
+  </si>
+  <si>
+    <t>Add automaps 485 (27x27, 92 bytes), 486 (11x19, 27 bytes), 487 (17x17, 37 bytes) and 488 (21x21, 56 bytes). They were missing in Save.00, entering 485/486 on the Amiga ends in a fatal error (Init_automap loads the entry for every 3D map).</t>
   </si>
 </sst>
 </file>
@@ -7755,17 +7755,17 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="27" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="21" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="27" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="21" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -10007,7 +10007,7 @@
         <v>911</v>
       </c>
       <c r="D48" t="s">
-        <v>2287</v>
+        <v>2286</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
@@ -10015,13 +10015,13 @@
         <v>488</v>
       </c>
       <c r="B49" t="s">
-        <v>2303</v>
+        <v>2302</v>
       </c>
       <c r="C49" t="s">
         <v>911</v>
       </c>
       <c r="D49" t="s">
-        <v>2304</v>
+        <v>2303</v>
       </c>
     </row>
   </sheetData>
@@ -10238,7 +10238,7 @@
         <v>46</v>
       </c>
       <c r="B14" t="s">
-        <v>2302</v>
+        <v>2301</v>
       </c>
     </row>
   </sheetData>
@@ -15030,10 +15030,10 @@
         <v>193</v>
       </c>
       <c r="B22" t="s">
+        <v>2287</v>
+      </c>
+      <c r="C22" t="s">
         <v>2288</v>
-      </c>
-      <c r="C22" t="s">
-        <v>2289</v>
       </c>
       <c r="D22" t="s">
         <v>1530</v>
@@ -15044,10 +15044,10 @@
         <v>194</v>
       </c>
       <c r="B23" t="s">
-        <v>2290</v>
+        <v>2289</v>
       </c>
       <c r="C23" t="s">
-        <v>2289</v>
+        <v>2288</v>
       </c>
       <c r="D23" t="s">
         <v>1530</v>
@@ -15058,10 +15058,10 @@
         <v>195</v>
       </c>
       <c r="B24" t="s">
-        <v>2291</v>
+        <v>2290</v>
       </c>
       <c r="C24" t="s">
-        <v>2289</v>
+        <v>2288</v>
       </c>
       <c r="D24" t="s">
         <v>1530</v>
@@ -15072,10 +15072,10 @@
         <v>196</v>
       </c>
       <c r="B25" t="s">
-        <v>2292</v>
+        <v>2291</v>
       </c>
       <c r="C25" t="s">
-        <v>2289</v>
+        <v>2288</v>
       </c>
       <c r="D25" t="s">
         <v>1530</v>
@@ -15086,10 +15086,10 @@
         <v>197</v>
       </c>
       <c r="B26" t="s">
-        <v>2293</v>
+        <v>2292</v>
       </c>
       <c r="C26" t="s">
-        <v>2289</v>
+        <v>2288</v>
       </c>
       <c r="D26" t="s">
         <v>1530</v>
@@ -15100,10 +15100,10 @@
         <v>198</v>
       </c>
       <c r="B27" t="s">
-        <v>2294</v>
+        <v>2293</v>
       </c>
       <c r="C27" t="s">
-        <v>2289</v>
+        <v>2288</v>
       </c>
       <c r="D27" t="s">
         <v>1530</v>
@@ -15114,10 +15114,10 @@
         <v>199</v>
       </c>
       <c r="B28" t="s">
-        <v>2295</v>
+        <v>2294</v>
       </c>
       <c r="C28" t="s">
-        <v>2289</v>
+        <v>2288</v>
       </c>
       <c r="D28" t="s">
         <v>1530</v>
@@ -15128,10 +15128,10 @@
         <v>200</v>
       </c>
       <c r="B29" t="s">
-        <v>2296</v>
+        <v>2295</v>
       </c>
       <c r="C29" t="s">
-        <v>2289</v>
+        <v>2288</v>
       </c>
       <c r="D29" t="s">
         <v>1530</v>
@@ -16005,10 +16005,10 @@
         <v>151</v>
       </c>
       <c r="B61" t="s">
-        <v>2297</v>
+        <v>2296</v>
       </c>
       <c r="C61" t="s">
-        <v>2289</v>
+        <v>2288</v>
       </c>
       <c r="D61" t="s">
         <v>1558</v>
@@ -16019,10 +16019,10 @@
         <v>152</v>
       </c>
       <c r="B62" t="s">
-        <v>2298</v>
+        <v>2297</v>
       </c>
       <c r="C62" t="s">
-        <v>2289</v>
+        <v>2288</v>
       </c>
       <c r="D62" t="s">
         <v>1558</v>
@@ -16033,10 +16033,10 @@
         <v>153</v>
       </c>
       <c r="B63" t="s">
-        <v>2299</v>
+        <v>2298</v>
       </c>
       <c r="C63" t="s">
-        <v>2289</v>
+        <v>2288</v>
       </c>
       <c r="D63" t="s">
         <v>1558</v>
@@ -16047,10 +16047,10 @@
         <v>154</v>
       </c>
       <c r="B64" t="s">
-        <v>2300</v>
+        <v>2299</v>
       </c>
       <c r="C64" t="s">
-        <v>2289</v>
+        <v>2288</v>
       </c>
       <c r="D64" t="s">
         <v>1558</v>
@@ -16061,10 +16061,10 @@
         <v>155</v>
       </c>
       <c r="B65" t="s">
-        <v>2301</v>
+        <v>2300</v>
       </c>
       <c r="C65" t="s">
-        <v>2289</v>
+        <v>2288</v>
       </c>
       <c r="D65" t="s">
         <v>1558</v>
@@ -17371,14 +17371,14 @@
       <c r="B32" s="54" t="s">
         <v>1745</v>
       </c>
-      <c r="C32" s="75" t="s">
+      <c r="C32" s="78" t="s">
         <v>1746</v>
       </c>
-      <c r="D32" s="75"/>
-      <c r="E32" s="75"/>
-      <c r="F32" s="75"/>
-      <c r="G32" s="75"/>
-      <c r="H32" s="75"/>
+      <c r="D32" s="78"/>
+      <c r="E32" s="78"/>
+      <c r="F32" s="78"/>
+      <c r="G32" s="78"/>
+      <c r="H32" s="78"/>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" s="36" t="s">
@@ -17387,14 +17387,14 @@
       <c r="B33" s="28" t="s">
         <v>1748</v>
       </c>
-      <c r="C33" s="76" t="s">
+      <c r="C33" s="77" t="s">
         <v>1749</v>
       </c>
-      <c r="D33" s="76"/>
-      <c r="E33" s="76"/>
-      <c r="F33" s="76"/>
-      <c r="G33" s="76"/>
-      <c r="H33" s="76"/>
+      <c r="D33" s="77"/>
+      <c r="E33" s="77"/>
+      <c r="F33" s="77"/>
+      <c r="G33" s="77"/>
+      <c r="H33" s="77"/>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" s="36" t="s">
@@ -17403,14 +17403,14 @@
       <c r="B34" s="28" t="s">
         <v>1748</v>
       </c>
-      <c r="C34" s="76" t="s">
+      <c r="C34" s="77" t="s">
         <v>1749</v>
       </c>
-      <c r="D34" s="76"/>
-      <c r="E34" s="76"/>
-      <c r="F34" s="76"/>
-      <c r="G34" s="76"/>
-      <c r="H34" s="76"/>
+      <c r="D34" s="77"/>
+      <c r="E34" s="77"/>
+      <c r="F34" s="77"/>
+      <c r="G34" s="77"/>
+      <c r="H34" s="77"/>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" s="36" t="s">
@@ -17419,14 +17419,14 @@
       <c r="B35" s="28" t="s">
         <v>1748</v>
       </c>
-      <c r="C35" s="76" t="s">
+      <c r="C35" s="77" t="s">
         <v>1749</v>
       </c>
-      <c r="D35" s="76"/>
-      <c r="E35" s="76"/>
-      <c r="F35" s="76"/>
-      <c r="G35" s="76"/>
-      <c r="H35" s="76"/>
+      <c r="D35" s="77"/>
+      <c r="E35" s="77"/>
+      <c r="F35" s="77"/>
+      <c r="G35" s="77"/>
+      <c r="H35" s="77"/>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" s="36" t="s">
@@ -17435,14 +17435,14 @@
       <c r="B36" s="28" t="s">
         <v>1734</v>
       </c>
-      <c r="C36" s="77" t="s">
+      <c r="C36" s="76" t="s">
         <v>1753</v>
       </c>
-      <c r="D36" s="77"/>
-      <c r="E36" s="77"/>
-      <c r="F36" s="77"/>
-      <c r="G36" s="77"/>
-      <c r="H36" s="77"/>
+      <c r="D36" s="76"/>
+      <c r="E36" s="76"/>
+      <c r="F36" s="76"/>
+      <c r="G36" s="76"/>
+      <c r="H36" s="76"/>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" s="36" t="s">
@@ -17451,14 +17451,14 @@
       <c r="B37" s="28" t="s">
         <v>1736</v>
       </c>
-      <c r="C37" s="76" t="s">
+      <c r="C37" s="77" t="s">
         <v>1755</v>
       </c>
-      <c r="D37" s="76"/>
-      <c r="E37" s="76"/>
-      <c r="F37" s="76"/>
-      <c r="G37" s="76"/>
-      <c r="H37" s="76"/>
+      <c r="D37" s="77"/>
+      <c r="E37" s="77"/>
+      <c r="F37" s="77"/>
+      <c r="G37" s="77"/>
+      <c r="H37" s="77"/>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" s="36" t="s">
@@ -17467,14 +17467,14 @@
       <c r="B38" s="28" t="s">
         <v>1734</v>
       </c>
-      <c r="C38" s="76" t="s">
+      <c r="C38" s="77" t="s">
         <v>1755</v>
       </c>
-      <c r="D38" s="76"/>
-      <c r="E38" s="76"/>
-      <c r="F38" s="76"/>
-      <c r="G38" s="76"/>
-      <c r="H38" s="76"/>
+      <c r="D38" s="77"/>
+      <c r="E38" s="77"/>
+      <c r="F38" s="77"/>
+      <c r="G38" s="77"/>
+      <c r="H38" s="77"/>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" s="36" t="s">
@@ -17483,14 +17483,14 @@
       <c r="B39" s="28" t="s">
         <v>1734</v>
       </c>
-      <c r="C39" s="77" t="s">
+      <c r="C39" s="76" t="s">
         <v>1753</v>
       </c>
-      <c r="D39" s="77"/>
-      <c r="E39" s="77"/>
-      <c r="F39" s="77"/>
-      <c r="G39" s="77"/>
-      <c r="H39" s="77"/>
+      <c r="D39" s="76"/>
+      <c r="E39" s="76"/>
+      <c r="F39" s="76"/>
+      <c r="G39" s="76"/>
+      <c r="H39" s="76"/>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" s="36" t="s">
@@ -17499,14 +17499,14 @@
       <c r="B40" s="28" t="s">
         <v>1734</v>
       </c>
-      <c r="C40" s="77" t="s">
+      <c r="C40" s="76" t="s">
         <v>1753</v>
       </c>
-      <c r="D40" s="77"/>
-      <c r="E40" s="77"/>
-      <c r="F40" s="77"/>
-      <c r="G40" s="77"/>
-      <c r="H40" s="77"/>
+      <c r="D40" s="76"/>
+      <c r="E40" s="76"/>
+      <c r="F40" s="76"/>
+      <c r="G40" s="76"/>
+      <c r="H40" s="76"/>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" s="36" t="s">
@@ -17515,14 +17515,14 @@
       <c r="B41" s="28" t="s">
         <v>1737</v>
       </c>
-      <c r="C41" s="77" t="s">
+      <c r="C41" s="76" t="s">
         <v>1759</v>
       </c>
-      <c r="D41" s="77"/>
-      <c r="E41" s="77"/>
-      <c r="F41" s="77"/>
-      <c r="G41" s="77"/>
-      <c r="H41" s="77"/>
+      <c r="D41" s="76"/>
+      <c r="E41" s="76"/>
+      <c r="F41" s="76"/>
+      <c r="G41" s="76"/>
+      <c r="H41" s="76"/>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" s="36" t="s">
@@ -17531,14 +17531,14 @@
       <c r="B42" s="28" t="s">
         <v>1738</v>
       </c>
-      <c r="C42" s="77" t="s">
+      <c r="C42" s="76" t="s">
         <v>1761</v>
       </c>
-      <c r="D42" s="77"/>
-      <c r="E42" s="77"/>
-      <c r="F42" s="77"/>
-      <c r="G42" s="77"/>
-      <c r="H42" s="77"/>
+      <c r="D42" s="76"/>
+      <c r="E42" s="76"/>
+      <c r="F42" s="76"/>
+      <c r="G42" s="76"/>
+      <c r="H42" s="76"/>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" s="36" t="s">
@@ -17547,14 +17547,14 @@
       <c r="B43" s="28" t="s">
         <v>1739</v>
       </c>
-      <c r="C43" s="77" t="s">
+      <c r="C43" s="76" t="s">
         <v>1763</v>
       </c>
-      <c r="D43" s="77"/>
-      <c r="E43" s="77"/>
-      <c r="F43" s="77"/>
-      <c r="G43" s="77"/>
-      <c r="H43" s="77"/>
+      <c r="D43" s="76"/>
+      <c r="E43" s="76"/>
+      <c r="F43" s="76"/>
+      <c r="G43" s="76"/>
+      <c r="H43" s="76"/>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" s="36" t="s">
@@ -17563,26 +17563,26 @@
       <c r="B44" s="28" t="s">
         <v>1740</v>
       </c>
-      <c r="C44" s="77" t="s">
+      <c r="C44" s="76" t="s">
         <v>1765</v>
       </c>
-      <c r="D44" s="77"/>
-      <c r="E44" s="77"/>
-      <c r="F44" s="77"/>
-      <c r="G44" s="77"/>
-      <c r="H44" s="77"/>
+      <c r="D44" s="76"/>
+      <c r="E44" s="76"/>
+      <c r="F44" s="76"/>
+      <c r="G44" s="76"/>
+      <c r="H44" s="76"/>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A48" s="78" t="s">
+      <c r="A48" s="75" t="s">
         <v>1754</v>
       </c>
-      <c r="B48" s="78"/>
-      <c r="C48" s="78"/>
-      <c r="D48" s="78"/>
-      <c r="E48" s="78"/>
-      <c r="F48" s="78"/>
-      <c r="G48" s="78"/>
-      <c r="H48" s="78"/>
+      <c r="B48" s="75"/>
+      <c r="C48" s="75"/>
+      <c r="D48" s="75"/>
+      <c r="E48" s="75"/>
+      <c r="F48" s="75"/>
+      <c r="G48" s="75"/>
+      <c r="H48" s="75"/>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
@@ -17595,16 +17595,16 @@
       </c>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A52" s="78" t="s">
+      <c r="A52" s="75" t="s">
         <v>1756</v>
       </c>
-      <c r="B52" s="78"/>
-      <c r="C52" s="78"/>
-      <c r="D52" s="78"/>
-      <c r="E52" s="78"/>
-      <c r="F52" s="78"/>
-      <c r="G52" s="78"/>
-      <c r="H52" s="78"/>
+      <c r="B52" s="75"/>
+      <c r="C52" s="75"/>
+      <c r="D52" s="75"/>
+      <c r="E52" s="75"/>
+      <c r="F52" s="75"/>
+      <c r="G52" s="75"/>
+      <c r="H52" s="75"/>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
@@ -17612,16 +17612,16 @@
       </c>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A57" s="78" t="s">
+      <c r="A57" s="75" t="s">
         <v>1769</v>
       </c>
-      <c r="B57" s="78"/>
-      <c r="C57" s="78"/>
-      <c r="D57" s="78"/>
-      <c r="E57" s="78"/>
-      <c r="F57" s="78"/>
-      <c r="G57" s="78"/>
-      <c r="H57" s="78"/>
+      <c r="B57" s="75"/>
+      <c r="C57" s="75"/>
+      <c r="D57" s="75"/>
+      <c r="E57" s="75"/>
+      <c r="F57" s="75"/>
+      <c r="G57" s="75"/>
+      <c r="H57" s="75"/>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
@@ -17689,12 +17689,12 @@
       </c>
     </row>
     <row r="73" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="H73" s="78" t="s">
+      <c r="H73" s="75" t="s">
         <v>1783</v>
       </c>
-      <c r="I73" s="78"/>
-      <c r="J73" s="78"/>
-      <c r="K73" s="78"/>
+      <c r="I73" s="75"/>
+      <c r="J73" s="75"/>
+      <c r="K73" s="75"/>
     </row>
     <row r="74" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A74" s="55" t="s">
@@ -18261,6 +18261,16 @@
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="C32:H32"/>
+    <mergeCell ref="C33:H33"/>
+    <mergeCell ref="C34:H34"/>
+    <mergeCell ref="C35:H35"/>
+    <mergeCell ref="C36:H36"/>
+    <mergeCell ref="C37:H37"/>
+    <mergeCell ref="C38:H38"/>
+    <mergeCell ref="C39:H39"/>
+    <mergeCell ref="C40:H40"/>
+    <mergeCell ref="C41:H41"/>
     <mergeCell ref="A57:H57"/>
     <mergeCell ref="H73:K73"/>
     <mergeCell ref="C42:H42"/>
@@ -18268,16 +18278,6 @@
     <mergeCell ref="C44:H44"/>
     <mergeCell ref="A48:H48"/>
     <mergeCell ref="A52:H52"/>
-    <mergeCell ref="C37:H37"/>
-    <mergeCell ref="C38:H38"/>
-    <mergeCell ref="C39:H39"/>
-    <mergeCell ref="C40:H40"/>
-    <mergeCell ref="C41:H41"/>
-    <mergeCell ref="C32:H32"/>
-    <mergeCell ref="C33:H33"/>
-    <mergeCell ref="C34:H34"/>
-    <mergeCell ref="C35:H35"/>
-    <mergeCell ref="C36:H36"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78749999999999998" bottom="0.78749999999999998" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -18340,13 +18340,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="78" t="s">
+      <c r="A1" s="75" t="s">
         <v>1905</v>
       </c>
-      <c r="B1" s="78"/>
-      <c r="C1" s="78"/>
-      <c r="D1" s="78"/>
-      <c r="E1" s="78"/>
+      <c r="B1" s="75"/>
+      <c r="C1" s="75"/>
+      <c r="D1" s="75"/>
+      <c r="E1" s="75"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="56" t="s">
@@ -18499,7 +18499,7 @@
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>2284</v>
+        <v>2304</v>
       </c>
     </row>
   </sheetData>
@@ -22685,10 +22685,10 @@
         <v>2282</v>
       </c>
       <c r="D34" t="s">
+        <v>2284</v>
+      </c>
+      <c r="E34" t="s">
         <v>2285</v>
-      </c>
-      <c r="E34" t="s">
-        <v>2286</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Amiga: events 28-32 (show map, toggle switch, dynamic tile change, rectangular exploration, vertical line reveal), event tables extended to 32
</commit_message>
<xml_diff>
--- a/AmbermoonAdvanced.xlsx
+++ b/AmbermoonAdvanced.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Robert\source\repos\Ambermoon-Advanced\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E632F1ED-ED07-4862-B11B-A4827A9C717A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32AA3BA8-3A52-4DA6-8E91-ED082C584105}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="500" firstSheet="39" activeTab="42" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -78,7 +78,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3232" uniqueCount="2312">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3248" uniqueCount="2324">
   <si>
     <t>Map texts</t>
   </si>
@@ -7131,6 +7131,42 @@
   </si>
   <si>
     <t>Lava tiles 235-238 block walking and the horse. Green slime (labdata 2 objects 15-17) passable for monsters (2026-10-18)</t>
+  </si>
+  <si>
+    <t>Delay</t>
+  </si>
+  <si>
+    <t>Amiga: yes</t>
+  </si>
+  <si>
+    <t>Party member condition</t>
+  </si>
+  <si>
+    <t>Shake</t>
+  </si>
+  <si>
+    <t>Show map</t>
+  </si>
+  <si>
+    <t>Amiga: implemented 2026-10-18 (was a savegame upgrade placeholder)</t>
+  </si>
+  <si>
+    <t>Toggle switch</t>
+  </si>
+  <si>
+    <t>Amiga: implemented 2026-10-18</t>
+  </si>
+  <si>
+    <t>Dynamic tile change</t>
+  </si>
+  <si>
+    <t>Rectangular exploration</t>
+  </si>
+  <si>
+    <t>Amiga: implemented 2026-10-18 (current map only)</t>
+  </si>
+  <si>
+    <t>Vertical line reveal</t>
   </si>
 </sst>
 </file>
@@ -7776,17 +7812,17 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="27" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="21" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="27" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="21" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -17436,14 +17472,14 @@
       <c r="B32" s="54" t="s">
         <v>1745</v>
       </c>
-      <c r="C32" s="75" t="s">
+      <c r="C32" s="78" t="s">
         <v>1746</v>
       </c>
-      <c r="D32" s="75"/>
-      <c r="E32" s="75"/>
-      <c r="F32" s="75"/>
-      <c r="G32" s="75"/>
-      <c r="H32" s="75"/>
+      <c r="D32" s="78"/>
+      <c r="E32" s="78"/>
+      <c r="F32" s="78"/>
+      <c r="G32" s="78"/>
+      <c r="H32" s="78"/>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A33" s="36" t="s">
@@ -17452,14 +17488,14 @@
       <c r="B33" s="28" t="s">
         <v>1748</v>
       </c>
-      <c r="C33" s="76" t="s">
+      <c r="C33" s="77" t="s">
         <v>1749</v>
       </c>
-      <c r="D33" s="76"/>
-      <c r="E33" s="76"/>
-      <c r="F33" s="76"/>
-      <c r="G33" s="76"/>
-      <c r="H33" s="76"/>
+      <c r="D33" s="77"/>
+      <c r="E33" s="77"/>
+      <c r="F33" s="77"/>
+      <c r="G33" s="77"/>
+      <c r="H33" s="77"/>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A34" s="36" t="s">
@@ -17468,14 +17504,14 @@
       <c r="B34" s="28" t="s">
         <v>1748</v>
       </c>
-      <c r="C34" s="76" t="s">
+      <c r="C34" s="77" t="s">
         <v>1749</v>
       </c>
-      <c r="D34" s="76"/>
-      <c r="E34" s="76"/>
-      <c r="F34" s="76"/>
-      <c r="G34" s="76"/>
-      <c r="H34" s="76"/>
+      <c r="D34" s="77"/>
+      <c r="E34" s="77"/>
+      <c r="F34" s="77"/>
+      <c r="G34" s="77"/>
+      <c r="H34" s="77"/>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A35" s="36" t="s">
@@ -17484,14 +17520,14 @@
       <c r="B35" s="28" t="s">
         <v>1748</v>
       </c>
-      <c r="C35" s="76" t="s">
+      <c r="C35" s="77" t="s">
         <v>1749</v>
       </c>
-      <c r="D35" s="76"/>
-      <c r="E35" s="76"/>
-      <c r="F35" s="76"/>
-      <c r="G35" s="76"/>
-      <c r="H35" s="76"/>
+      <c r="D35" s="77"/>
+      <c r="E35" s="77"/>
+      <c r="F35" s="77"/>
+      <c r="G35" s="77"/>
+      <c r="H35" s="77"/>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A36" s="36" t="s">
@@ -17500,14 +17536,14 @@
       <c r="B36" s="28" t="s">
         <v>1734</v>
       </c>
-      <c r="C36" s="77" t="s">
+      <c r="C36" s="76" t="s">
         <v>1753</v>
       </c>
-      <c r="D36" s="77"/>
-      <c r="E36" s="77"/>
-      <c r="F36" s="77"/>
-      <c r="G36" s="77"/>
-      <c r="H36" s="77"/>
+      <c r="D36" s="76"/>
+      <c r="E36" s="76"/>
+      <c r="F36" s="76"/>
+      <c r="G36" s="76"/>
+      <c r="H36" s="76"/>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A37" s="36" t="s">
@@ -17516,14 +17552,14 @@
       <c r="B37" s="28" t="s">
         <v>1736</v>
       </c>
-      <c r="C37" s="76" t="s">
+      <c r="C37" s="77" t="s">
         <v>1755</v>
       </c>
-      <c r="D37" s="76"/>
-      <c r="E37" s="76"/>
-      <c r="F37" s="76"/>
-      <c r="G37" s="76"/>
-      <c r="H37" s="76"/>
+      <c r="D37" s="77"/>
+      <c r="E37" s="77"/>
+      <c r="F37" s="77"/>
+      <c r="G37" s="77"/>
+      <c r="H37" s="77"/>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A38" s="36" t="s">
@@ -17532,14 +17568,14 @@
       <c r="B38" s="28" t="s">
         <v>1734</v>
       </c>
-      <c r="C38" s="76" t="s">
+      <c r="C38" s="77" t="s">
         <v>1755</v>
       </c>
-      <c r="D38" s="76"/>
-      <c r="E38" s="76"/>
-      <c r="F38" s="76"/>
-      <c r="G38" s="76"/>
-      <c r="H38" s="76"/>
+      <c r="D38" s="77"/>
+      <c r="E38" s="77"/>
+      <c r="F38" s="77"/>
+      <c r="G38" s="77"/>
+      <c r="H38" s="77"/>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A39" s="36" t="s">
@@ -17548,14 +17584,14 @@
       <c r="B39" s="28" t="s">
         <v>1734</v>
       </c>
-      <c r="C39" s="77" t="s">
+      <c r="C39" s="76" t="s">
         <v>1753</v>
       </c>
-      <c r="D39" s="77"/>
-      <c r="E39" s="77"/>
-      <c r="F39" s="77"/>
-      <c r="G39" s="77"/>
-      <c r="H39" s="77"/>
+      <c r="D39" s="76"/>
+      <c r="E39" s="76"/>
+      <c r="F39" s="76"/>
+      <c r="G39" s="76"/>
+      <c r="H39" s="76"/>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A40" s="36" t="s">
@@ -17564,14 +17600,14 @@
       <c r="B40" s="28" t="s">
         <v>1734</v>
       </c>
-      <c r="C40" s="77" t="s">
+      <c r="C40" s="76" t="s">
         <v>1753</v>
       </c>
-      <c r="D40" s="77"/>
-      <c r="E40" s="77"/>
-      <c r="F40" s="77"/>
-      <c r="G40" s="77"/>
-      <c r="H40" s="77"/>
+      <c r="D40" s="76"/>
+      <c r="E40" s="76"/>
+      <c r="F40" s="76"/>
+      <c r="G40" s="76"/>
+      <c r="H40" s="76"/>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A41" s="36" t="s">
@@ -17580,14 +17616,14 @@
       <c r="B41" s="28" t="s">
         <v>1737</v>
       </c>
-      <c r="C41" s="77" t="s">
+      <c r="C41" s="76" t="s">
         <v>1759</v>
       </c>
-      <c r="D41" s="77"/>
-      <c r="E41" s="77"/>
-      <c r="F41" s="77"/>
-      <c r="G41" s="77"/>
-      <c r="H41" s="77"/>
+      <c r="D41" s="76"/>
+      <c r="E41" s="76"/>
+      <c r="F41" s="76"/>
+      <c r="G41" s="76"/>
+      <c r="H41" s="76"/>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A42" s="36" t="s">
@@ -17596,14 +17632,14 @@
       <c r="B42" s="28" t="s">
         <v>1738</v>
       </c>
-      <c r="C42" s="77" t="s">
+      <c r="C42" s="76" t="s">
         <v>1761</v>
       </c>
-      <c r="D42" s="77"/>
-      <c r="E42" s="77"/>
-      <c r="F42" s="77"/>
-      <c r="G42" s="77"/>
-      <c r="H42" s="77"/>
+      <c r="D42" s="76"/>
+      <c r="E42" s="76"/>
+      <c r="F42" s="76"/>
+      <c r="G42" s="76"/>
+      <c r="H42" s="76"/>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A43" s="36" t="s">
@@ -17612,14 +17648,14 @@
       <c r="B43" s="28" t="s">
         <v>1739</v>
       </c>
-      <c r="C43" s="77" t="s">
+      <c r="C43" s="76" t="s">
         <v>1763</v>
       </c>
-      <c r="D43" s="77"/>
-      <c r="E43" s="77"/>
-      <c r="F43" s="77"/>
-      <c r="G43" s="77"/>
-      <c r="H43" s="77"/>
+      <c r="D43" s="76"/>
+      <c r="E43" s="76"/>
+      <c r="F43" s="76"/>
+      <c r="G43" s="76"/>
+      <c r="H43" s="76"/>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A44" s="36" t="s">
@@ -17628,26 +17664,26 @@
       <c r="B44" s="28" t="s">
         <v>1740</v>
       </c>
-      <c r="C44" s="77" t="s">
+      <c r="C44" s="76" t="s">
         <v>1765</v>
       </c>
-      <c r="D44" s="77"/>
-      <c r="E44" s="77"/>
-      <c r="F44" s="77"/>
-      <c r="G44" s="77"/>
-      <c r="H44" s="77"/>
+      <c r="D44" s="76"/>
+      <c r="E44" s="76"/>
+      <c r="F44" s="76"/>
+      <c r="G44" s="76"/>
+      <c r="H44" s="76"/>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A48" s="78" t="s">
+      <c r="A48" s="75" t="s">
         <v>1754</v>
       </c>
-      <c r="B48" s="78"/>
-      <c r="C48" s="78"/>
-      <c r="D48" s="78"/>
-      <c r="E48" s="78"/>
-      <c r="F48" s="78"/>
-      <c r="G48" s="78"/>
-      <c r="H48" s="78"/>
+      <c r="B48" s="75"/>
+      <c r="C48" s="75"/>
+      <c r="D48" s="75"/>
+      <c r="E48" s="75"/>
+      <c r="F48" s="75"/>
+      <c r="G48" s="75"/>
+      <c r="H48" s="75"/>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
@@ -17660,16 +17696,16 @@
       </c>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A52" s="78" t="s">
+      <c r="A52" s="75" t="s">
         <v>1756</v>
       </c>
-      <c r="B52" s="78"/>
-      <c r="C52" s="78"/>
-      <c r="D52" s="78"/>
-      <c r="E52" s="78"/>
-      <c r="F52" s="78"/>
-      <c r="G52" s="78"/>
-      <c r="H52" s="78"/>
+      <c r="B52" s="75"/>
+      <c r="C52" s="75"/>
+      <c r="D52" s="75"/>
+      <c r="E52" s="75"/>
+      <c r="F52" s="75"/>
+      <c r="G52" s="75"/>
+      <c r="H52" s="75"/>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
@@ -17677,16 +17713,16 @@
       </c>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A57" s="78" t="s">
+      <c r="A57" s="75" t="s">
         <v>1769</v>
       </c>
-      <c r="B57" s="78"/>
-      <c r="C57" s="78"/>
-      <c r="D57" s="78"/>
-      <c r="E57" s="78"/>
-      <c r="F57" s="78"/>
-      <c r="G57" s="78"/>
-      <c r="H57" s="78"/>
+      <c r="B57" s="75"/>
+      <c r="C57" s="75"/>
+      <c r="D57" s="75"/>
+      <c r="E57" s="75"/>
+      <c r="F57" s="75"/>
+      <c r="G57" s="75"/>
+      <c r="H57" s="75"/>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
@@ -17754,12 +17790,12 @@
       </c>
     </row>
     <row r="73" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="H73" s="78" t="s">
+      <c r="H73" s="75" t="s">
         <v>1783</v>
       </c>
-      <c r="I73" s="78"/>
-      <c r="J73" s="78"/>
-      <c r="K73" s="78"/>
+      <c r="I73" s="75"/>
+      <c r="J73" s="75"/>
+      <c r="K73" s="75"/>
     </row>
     <row r="74" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A74" s="55" t="s">
@@ -18326,6 +18362,16 @@
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="C32:H32"/>
+    <mergeCell ref="C33:H33"/>
+    <mergeCell ref="C34:H34"/>
+    <mergeCell ref="C35:H35"/>
+    <mergeCell ref="C36:H36"/>
+    <mergeCell ref="C37:H37"/>
+    <mergeCell ref="C38:H38"/>
+    <mergeCell ref="C39:H39"/>
+    <mergeCell ref="C40:H40"/>
+    <mergeCell ref="C41:H41"/>
     <mergeCell ref="A57:H57"/>
     <mergeCell ref="H73:K73"/>
     <mergeCell ref="C42:H42"/>
@@ -18333,16 +18379,6 @@
     <mergeCell ref="C44:H44"/>
     <mergeCell ref="A48:H48"/>
     <mergeCell ref="A52:H52"/>
-    <mergeCell ref="C37:H37"/>
-    <mergeCell ref="C38:H38"/>
-    <mergeCell ref="C39:H39"/>
-    <mergeCell ref="C40:H40"/>
-    <mergeCell ref="C41:H41"/>
-    <mergeCell ref="C32:H32"/>
-    <mergeCell ref="C33:H33"/>
-    <mergeCell ref="C34:H34"/>
-    <mergeCell ref="C35:H35"/>
-    <mergeCell ref="C36:H36"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78749999999999998" bottom="0.78749999999999998" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -18405,13 +18441,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A1" s="78" t="s">
+      <c r="A1" s="75" t="s">
         <v>1905</v>
       </c>
-      <c r="B1" s="78"/>
-      <c r="C1" s="78"/>
-      <c r="D1" s="78"/>
-      <c r="E1" s="78"/>
+      <c r="B1" s="75"/>
+      <c r="C1" s="75"/>
+      <c r="D1" s="75"/>
+      <c r="E1" s="75"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" s="56" t="s">
@@ -18625,6 +18661,15 @@
       </c>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A3">
+        <v>25</v>
+      </c>
+      <c r="B3" t="s">
+        <v>2312</v>
+      </c>
+      <c r="C3" t="s">
+        <v>2313</v>
+      </c>
       <c r="E3">
         <v>22</v>
       </c>
@@ -18636,6 +18681,15 @@
       </c>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A4">
+        <v>26</v>
+      </c>
+      <c r="B4" t="s">
+        <v>2314</v>
+      </c>
+      <c r="C4" t="s">
+        <v>2313</v>
+      </c>
       <c r="E4">
         <v>23</v>
       </c>
@@ -18647,6 +18701,15 @@
       </c>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A5">
+        <v>27</v>
+      </c>
+      <c r="B5" t="s">
+        <v>2315</v>
+      </c>
+      <c r="C5" t="s">
+        <v>2313</v>
+      </c>
       <c r="E5">
         <v>24</v>
       </c>
@@ -18658,26 +18721,71 @@
       </c>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A6">
+        <v>28</v>
+      </c>
+      <c r="B6" t="s">
+        <v>2316</v>
+      </c>
+      <c r="C6" t="s">
+        <v>2317</v>
+      </c>
       <c r="I6" t="s">
         <v>1935</v>
       </c>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A7">
+        <v>29</v>
+      </c>
+      <c r="B7" t="s">
+        <v>2318</v>
+      </c>
+      <c r="C7" t="s">
+        <v>2319</v>
+      </c>
       <c r="I7" t="s">
         <v>1936</v>
       </c>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A8">
+        <v>30</v>
+      </c>
+      <c r="B8" t="s">
+        <v>2320</v>
+      </c>
+      <c r="C8" t="s">
+        <v>2319</v>
+      </c>
       <c r="I8" t="s">
         <v>1937</v>
       </c>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A9">
+        <v>31</v>
+      </c>
+      <c r="B9" t="s">
+        <v>2321</v>
+      </c>
+      <c r="C9" t="s">
+        <v>2322</v>
+      </c>
       <c r="I9" t="s">
         <v>1938</v>
       </c>
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A10">
+        <v>32</v>
+      </c>
+      <c r="B10" t="s">
+        <v>2323</v>
+      </c>
+      <c r="C10" t="s">
+        <v>2319</v>
+      </c>
       <c r="I10" t="s">
         <v>1939</v>
       </c>

</xml_diff>